<commit_message>
Initial commit of speech generation files
</commit_message>
<xml_diff>
--- a/SpeechGenerationAudit.xlsx
+++ b/SpeechGenerationAudit.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pc\Speech Generation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:2009_{46A8D271-2B1A-4D67-B90E-BF3339CA30E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:2009_{D06D5749-81B6-44F1-BA47-2C9F1558BB54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{A672C37D-E69E-470F-9024-46D64C3F6E80}"/>
+    <workbookView xWindow="444" yWindow="3204" windowWidth="11808" windowHeight="9960" activeTab="1" xr2:uid="{A672C37D-E69E-470F-9024-46D64C3F6E80}"/>
   </bookViews>
   <sheets>
     <sheet name="Audio + String Table " sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="689" uniqueCount="313">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="690" uniqueCount="323">
   <si>
     <t>Unity Key</t>
   </si>
@@ -310,9 +310,6 @@
     <t>Oh! that's nice to hear, Let's train!</t>
   </si>
   <si>
-    <t xml:space="preserve">Sounds a little robotic </t>
-  </si>
-  <si>
     <t>Unity Spanish Text</t>
   </si>
   <si>
@@ -715,9 +712,6 @@
     <t>அருமை! நாம ரெண்டு பேரும் சேர்ந்து மகிழலாம்!</t>
   </si>
   <si>
-    <t>No audio</t>
-  </si>
-  <si>
     <t>Unity Thai Text</t>
   </si>
   <si>
@@ -980,13 +974,49 @@
   </si>
   <si>
     <t xml:space="preserve">Audio does not match (same as German)                                   </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fixed </t>
+  </si>
+  <si>
+    <t xml:space="preserve">There is Norwegian audio, but not Norwegian text. </t>
+  </si>
+  <si>
+    <t>No audio : FIXED</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No audio: Buka kunci item yang dipilih? - FIXED </t>
+  </si>
+  <si>
+    <t>No audio : Awak nak berhenti kerja ke ? - FIXED</t>
+  </si>
+  <si>
+    <t>No audio: Anda tidak mempun yai syiling yang mencukupi - FIXED</t>
+  </si>
+  <si>
+    <t>No audio: தேர்ந்தெடுத்த பொருளை திறக்கவா? - FIXED</t>
+  </si>
+  <si>
+    <t>No audio: நீங்க வெளியேறணுமா? - FIXED</t>
+  </si>
+  <si>
+    <t>No audio: உங்களிடம் போதுமான நாணயங்கள் இல்லை. - FIXED</t>
+  </si>
+  <si>
+    <t>No audio: ปลดล็อกรายการที่เลือกใช่หรือไม่? - FIXED</t>
+  </si>
+  <si>
+    <t>No audio: คุณต้องการลาออกหรือไม่? - FIXED</t>
+  </si>
+  <si>
+    <t>No audio : คุณมีเหรียญไม่พอ - FIXED</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1037,6 +1067,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="9"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -1073,7 +1110,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
@@ -1135,6 +1172,10 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1534,19 +1575,19 @@
         <v>2</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>3</v>
@@ -1570,115 +1611,115 @@
         <v>3</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="P1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="R1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="T1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="V1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="X1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="Y1" s="1" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="Z1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="AA1" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="AB1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="AC1" s="1" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="AD1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="AE1" s="1" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="AF1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="AG1" s="1" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="AH1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="AI1" s="1" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="AJ1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="AK1" s="1" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="AL1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="AM1" s="1" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="AN1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="AO1" s="1" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="AP1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="AQ1" s="1" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="AR1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="AS1" s="1" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="AT1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="AU1" s="1" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="AV1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="AW1" s="1" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="AX1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="AY1" s="1" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="AZ1" s="1" t="s">
         <v>3</v>
@@ -1692,25 +1733,25 @@
         <v>63</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="D2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="F2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="G2" s="9" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="H2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="I2" s="9" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="J2" s="10" t="s">
         <v>56</v>
@@ -1728,115 +1769,115 @@
         <v>56</v>
       </c>
       <c r="O2" s="9" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="P2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="Q2" s="9" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="R2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="S2" s="9" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="T2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="U2" s="9" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="V2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="W2" s="9" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="X2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="Y2" s="9" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="Z2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AA2" s="9" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="AB2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AC2" s="9" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="AD2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AE2" s="18" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="AF2" s="19" t="s">
-        <v>164</v>
+        <v>313</v>
       </c>
       <c r="AG2" s="9" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="AH2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AI2" s="9" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="AJ2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AK2" s="9" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="AL2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AM2" s="9" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="AN2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AO2" s="9" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="AP2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AQ2" s="9" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AR2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AS2" s="18" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="AT2" s="19" t="s">
+        <v>313</v>
+      </c>
+      <c r="AU2" s="18" t="s">
         <v>224</v>
       </c>
-      <c r="AU2" s="18" t="s">
-        <v>226</v>
-      </c>
       <c r="AV2" s="19" t="s">
-        <v>164</v>
+        <v>313</v>
       </c>
       <c r="AW2" s="9" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="AX2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AY2" s="9" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="AZ2" s="10" t="s">
         <v>56</v>
@@ -1850,25 +1891,25 @@
         <v>64</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="D3" s="10" t="s">
         <v>56</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="F3" s="10" t="s">
         <v>56</v>
       </c>
       <c r="G3" s="9" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="H3" s="10" t="s">
         <v>56</v>
       </c>
       <c r="I3" s="9" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="J3" s="10" t="s">
         <v>56</v>
@@ -1886,115 +1927,115 @@
         <v>56</v>
       </c>
       <c r="O3" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="P3" s="10" t="s">
         <v>56</v>
       </c>
       <c r="Q3" s="9" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="R3" s="10" t="s">
         <v>56</v>
       </c>
       <c r="S3" s="9" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="T3" s="10" t="s">
         <v>56</v>
       </c>
       <c r="U3" s="9" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="V3" s="10" t="s">
         <v>56</v>
       </c>
       <c r="W3" s="9" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="X3" s="10" t="s">
         <v>56</v>
       </c>
       <c r="Y3" s="9" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="Z3" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AA3" s="9" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="AB3" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AC3" s="9" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="AD3" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AE3" s="18" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="AF3" s="19" t="s">
-        <v>164</v>
+        <v>313</v>
       </c>
       <c r="AG3" s="9" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="AH3" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AI3" s="9" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="AJ3" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AK3" s="9" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AL3" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AM3" s="9" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="AN3" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AO3" s="9" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="AP3" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AQ3" s="9" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="AR3" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AS3" s="18" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="AT3" s="19" t="s">
-        <v>224</v>
+        <v>313</v>
       </c>
       <c r="AU3" s="18" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="AV3" s="19" t="s">
-        <v>164</v>
+        <v>313</v>
       </c>
       <c r="AW3" s="9" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="AX3" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AY3" s="9" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="AZ3" s="10" t="s">
         <v>56</v>
@@ -2008,25 +2049,25 @@
         <v>60</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="D4" s="10" t="s">
         <v>56</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="F4" s="10" t="s">
         <v>56</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="H4" s="10" t="s">
         <v>56</v>
       </c>
       <c r="I4" s="9" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="J4" s="10" t="s">
         <v>56</v>
@@ -2037,122 +2078,122 @@
       <c r="L4" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="M4" s="16" t="s">
+      <c r="M4" s="23" t="s">
         <v>86</v>
       </c>
-      <c r="N4" s="17" t="s">
-        <v>89</v>
+      <c r="N4" s="24" t="s">
+        <v>311</v>
       </c>
       <c r="O4" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="P4" s="10" t="s">
         <v>56</v>
       </c>
       <c r="Q4" s="16" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="R4" s="16" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="S4" s="9" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="T4" s="10" t="s">
         <v>56</v>
       </c>
       <c r="U4" s="9" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="V4" s="10" t="s">
         <v>56</v>
       </c>
       <c r="W4" s="9" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="X4" s="10" t="s">
         <v>56</v>
       </c>
       <c r="Y4" s="9" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Z4" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AA4" s="9" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="AB4" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AC4" s="9" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="AD4" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AE4" s="18" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="AF4" s="19" t="s">
-        <v>164</v>
+        <v>313</v>
       </c>
       <c r="AG4" s="9" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="AH4" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AI4" s="9" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="AJ4" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AK4" s="9" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="AL4" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AM4" s="16" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="AN4" s="17" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="AO4" s="9" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="AP4" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AQ4" s="9" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="AR4" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AS4" s="18" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="AT4" s="19" t="s">
-        <v>224</v>
+        <v>313</v>
       </c>
       <c r="AU4" s="18" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="AV4" s="19" t="s">
-        <v>164</v>
+        <v>313</v>
       </c>
       <c r="AW4" s="9" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="AX4" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AY4" s="9" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="AZ4" s="10" t="s">
         <v>56</v>
@@ -2166,25 +2207,25 @@
         <v>57</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="D5" s="10" t="s">
         <v>56</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="F5" s="10" t="s">
         <v>56</v>
       </c>
       <c r="G5" s="9" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="H5" s="10" t="s">
         <v>56</v>
       </c>
       <c r="I5" s="9" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="J5" s="10" t="s">
         <v>56</v>
@@ -2195,122 +2236,122 @@
       <c r="L5" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="M5" s="16" t="s">
+      <c r="M5" s="23" t="s">
         <v>87</v>
       </c>
-      <c r="N5" s="17" t="s">
-        <v>89</v>
+      <c r="N5" s="24" t="s">
+        <v>311</v>
       </c>
       <c r="O5" s="9" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="P5" s="10" t="s">
         <v>56</v>
       </c>
       <c r="Q5" s="9" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="R5" s="10" t="s">
         <v>56</v>
       </c>
       <c r="S5" s="9" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="T5" s="10" t="s">
         <v>56</v>
       </c>
       <c r="U5" s="9" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="V5" s="10" t="s">
         <v>56</v>
       </c>
       <c r="W5" s="9" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="X5" s="10" t="s">
         <v>56</v>
       </c>
       <c r="Y5" s="9" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="Z5" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AA5" s="16" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="AB5" s="16" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="AC5" s="9" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="AD5" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AE5" s="18" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="AF5" s="19" t="s">
-        <v>164</v>
+        <v>313</v>
       </c>
       <c r="AG5" s="9" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="AH5" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AI5" s="9" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="AJ5" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AK5" s="9" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="AL5" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AM5" s="16" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="AN5" s="16" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="AO5" s="9" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="AP5" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AQ5" s="9" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="AR5" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AS5" s="18" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="AT5" s="19" t="s">
-        <v>224</v>
+        <v>313</v>
       </c>
       <c r="AU5" s="18" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="AV5" s="19" t="s">
-        <v>164</v>
+        <v>313</v>
       </c>
       <c r="AW5" s="9" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="AX5" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AY5" s="9" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="AZ5" s="10" t="s">
         <v>56</v>
@@ -2324,28 +2365,28 @@
         <v>58</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="D6" s="10" t="s">
         <v>59</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="F6" s="10" t="s">
         <v>59</v>
       </c>
       <c r="G6" s="9" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="H6" s="10" t="s">
         <v>59</v>
       </c>
       <c r="I6" s="9" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="J6" s="10" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="K6" s="9" t="s">
         <v>34</v>
@@ -2360,115 +2401,115 @@
         <v>59</v>
       </c>
       <c r="O6" s="9" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="P6" s="10" t="s">
         <v>59</v>
       </c>
       <c r="Q6" s="9" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="R6" s="10" t="s">
         <v>59</v>
       </c>
       <c r="S6" s="9" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="T6" s="10" t="s">
         <v>59</v>
       </c>
       <c r="U6" s="9" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="V6" s="10" t="s">
         <v>59</v>
       </c>
       <c r="W6" s="9" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="X6" s="10" t="s">
         <v>59</v>
       </c>
       <c r="Y6" s="9" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="Z6" s="10" t="s">
         <v>59</v>
       </c>
       <c r="AA6" s="16" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="AB6" s="16" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="AC6" s="9" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="AD6" s="10" t="s">
         <v>59</v>
       </c>
       <c r="AE6" s="18" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="AF6" s="19" t="s">
-        <v>164</v>
+        <v>313</v>
       </c>
       <c r="AG6" s="9" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="AH6" s="10" t="s">
         <v>59</v>
       </c>
       <c r="AI6" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="AJ6" s="10" t="s">
         <v>59</v>
       </c>
       <c r="AK6" s="9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="AL6" s="10" t="s">
         <v>59</v>
       </c>
       <c r="AM6" s="9" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="AN6" s="10" t="s">
         <v>59</v>
       </c>
       <c r="AO6" s="9" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="AP6" s="10" t="s">
         <v>59</v>
       </c>
       <c r="AQ6" s="9" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="AR6" s="10" t="s">
         <v>59</v>
       </c>
       <c r="AS6" s="18" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="AT6" s="19" t="s">
-        <v>224</v>
+        <v>313</v>
       </c>
       <c r="AU6" s="18" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="AV6" s="19" t="s">
-        <v>164</v>
+        <v>313</v>
       </c>
       <c r="AW6" s="9" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="AX6" s="10" t="s">
         <v>59</v>
       </c>
       <c r="AY6" s="9" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="AZ6" s="10" t="s">
         <v>59</v>
@@ -2482,25 +2523,25 @@
         <v>61</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="D7" s="10" t="s">
         <v>56</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="F7" s="10" t="s">
         <v>56</v>
       </c>
       <c r="G7" s="9" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="H7" s="10" t="s">
         <v>56</v>
       </c>
       <c r="I7" s="9" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="J7" s="10" t="s">
         <v>56</v>
@@ -2518,115 +2559,115 @@
         <v>56</v>
       </c>
       <c r="O7" s="9" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="P7" s="10" t="s">
         <v>56</v>
       </c>
       <c r="Q7" s="16" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="R7" s="16" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="S7" s="9" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="T7" s="10" t="s">
         <v>56</v>
       </c>
       <c r="U7" s="9" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="V7" s="10" t="s">
         <v>56</v>
       </c>
       <c r="W7" s="9" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="X7" s="10" t="s">
         <v>56</v>
       </c>
       <c r="Y7" s="9" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="Z7" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AA7" s="16" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="AB7" s="16" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="AC7" s="9" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="AD7" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AE7" s="18" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="AF7" s="19" t="s">
-        <v>164</v>
+        <v>313</v>
       </c>
       <c r="AG7" s="9" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="AH7" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AI7" s="9" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="AJ7" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AK7" s="9" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="AL7" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AM7" s="16" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="AN7" s="17" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="AO7" s="9" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="AP7" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AQ7" s="9" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="AR7" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AS7" s="18" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="AT7" s="19" t="s">
-        <v>224</v>
+        <v>313</v>
       </c>
       <c r="AU7" s="18" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="AV7" s="19" t="s">
-        <v>164</v>
+        <v>313</v>
       </c>
       <c r="AW7" s="9" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="AX7" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AY7" s="9" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="AZ7" s="10" t="s">
         <v>56</v>
@@ -2640,25 +2681,25 @@
         <v>62</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="D8" s="10" t="s">
         <v>56</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="F8" s="10" t="s">
         <v>56</v>
       </c>
       <c r="G8" s="9" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="H8" s="10" t="s">
         <v>56</v>
       </c>
       <c r="I8" s="9" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="J8" s="10" t="s">
         <v>56</v>
@@ -2676,115 +2717,115 @@
         <v>56</v>
       </c>
       <c r="O8" s="9" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="P8" s="10" t="s">
         <v>56</v>
       </c>
       <c r="Q8" s="9" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="R8" s="10" t="s">
         <v>56</v>
       </c>
       <c r="S8" s="9" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="T8" s="10" t="s">
         <v>56</v>
       </c>
       <c r="U8" s="9" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="V8" s="10" t="s">
         <v>56</v>
       </c>
       <c r="W8" s="9" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="X8" s="10" t="s">
         <v>56</v>
       </c>
       <c r="Y8" s="9" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="Z8" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AA8" s="9" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="AB8" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AC8" s="9" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="AD8" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AE8" s="18" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="AF8" s="19" t="s">
-        <v>164</v>
+        <v>313</v>
       </c>
       <c r="AG8" s="9" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="AH8" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AI8" s="9" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="AJ8" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AK8" s="9" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="AL8" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AM8" s="9" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="AN8" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AO8" s="9" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="AP8" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AQ8" s="9" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="AR8" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AS8" s="18" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="AT8" s="19" t="s">
-        <v>224</v>
+        <v>313</v>
       </c>
       <c r="AU8" s="18" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="AV8" s="19" t="s">
-        <v>164</v>
+        <v>313</v>
       </c>
       <c r="AW8" s="9" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="AX8" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AY8" s="9" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="AZ8" s="10" t="s">
         <v>56</v>
@@ -2845,6 +2886,9 @@
       <c r="J11" s="3"/>
       <c r="K11" s="3" t="s">
         <v>39</v>
+      </c>
+      <c r="AL11" s="19" t="s">
+        <v>312</v>
       </c>
     </row>
     <row r="12" spans="1:52" x14ac:dyDescent="0.3">
@@ -3200,15 +3244,16 @@
     <col min="14" max="14" width="26.44140625" customWidth="1"/>
     <col min="15" max="15" width="28.5546875" customWidth="1"/>
     <col min="16" max="16" width="26.33203125" customWidth="1"/>
-    <col min="17" max="17" width="26.44140625" customWidth="1"/>
+    <col min="17" max="17" width="38.88671875" customWidth="1"/>
     <col min="18" max="18" width="27.109375" customWidth="1"/>
     <col min="19" max="19" width="26.6640625" customWidth="1"/>
     <col min="20" max="20" width="31.33203125" customWidth="1"/>
     <col min="21" max="21" width="27.44140625" customWidth="1"/>
     <col min="22" max="22" width="25.77734375" customWidth="1"/>
     <col min="23" max="23" width="27.77734375" customWidth="1"/>
-    <col min="24" max="24" width="25.5546875" customWidth="1"/>
-    <col min="25" max="26" width="25.21875" customWidth="1"/>
+    <col min="24" max="24" width="44.6640625" customWidth="1"/>
+    <col min="25" max="25" width="45.5546875" customWidth="1"/>
+    <col min="26" max="26" width="25.21875" customWidth="1"/>
     <col min="27" max="27" width="26.6640625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -3220,79 +3265,79 @@
         <v>67</v>
       </c>
       <c r="C1" s="6" t="s">
+        <v>279</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>280</v>
+      </c>
+      <c r="E1" s="6" t="s">
         <v>281</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="F1" s="6" t="s">
         <v>282</v>
-      </c>
-      <c r="E1" s="6" t="s">
-        <v>283</v>
-      </c>
-      <c r="F1" s="6" t="s">
-        <v>284</v>
       </c>
       <c r="G1" s="6" t="s">
         <v>68</v>
       </c>
       <c r="H1" s="6" t="s">
+        <v>283</v>
+      </c>
+      <c r="I1" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="J1" s="6" t="s">
         <v>285</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="K1" s="6" t="s">
         <v>286</v>
       </c>
-      <c r="J1" s="6" t="s">
+      <c r="L1" s="6" t="s">
         <v>287</v>
       </c>
-      <c r="K1" s="6" t="s">
+      <c r="M1" s="6" t="s">
         <v>288</v>
       </c>
-      <c r="L1" s="6" t="s">
+      <c r="N1" s="6" t="s">
         <v>289</v>
       </c>
-      <c r="M1" s="6" t="s">
+      <c r="O1" s="6" t="s">
         <v>290</v>
       </c>
-      <c r="N1" s="6" t="s">
+      <c r="P1" s="6" t="s">
         <v>291</v>
       </c>
-      <c r="O1" s="6" t="s">
+      <c r="Q1" s="6" t="s">
         <v>292</v>
       </c>
-      <c r="P1" s="6" t="s">
+      <c r="R1" s="6" t="s">
         <v>293</v>
       </c>
-      <c r="Q1" s="6" t="s">
+      <c r="S1" s="6" t="s">
         <v>294</v>
       </c>
-      <c r="R1" s="6" t="s">
+      <c r="T1" s="6" t="s">
         <v>295</v>
       </c>
-      <c r="S1" s="6" t="s">
+      <c r="U1" s="6" t="s">
         <v>296</v>
       </c>
-      <c r="T1" s="6" t="s">
+      <c r="V1" s="6" t="s">
         <v>297</v>
       </c>
-      <c r="U1" s="6" t="s">
+      <c r="W1" s="6" t="s">
         <v>298</v>
       </c>
-      <c r="V1" s="6" t="s">
+      <c r="X1" s="6" t="s">
         <v>299</v>
       </c>
-      <c r="W1" s="6" t="s">
+      <c r="Y1" s="6" t="s">
         <v>300</v>
       </c>
-      <c r="X1" s="6" t="s">
+      <c r="Z1" s="6" t="s">
         <v>301</v>
       </c>
-      <c r="Y1" s="6" t="s">
+      <c r="AA1" s="6" t="s">
         <v>302</v>
-      </c>
-      <c r="Z1" s="6" t="s">
-        <v>303</v>
-      </c>
-      <c r="AA1" s="6" t="s">
-        <v>304</v>
       </c>
       <c r="AB1" s="6"/>
       <c r="AC1" s="6"/>
@@ -3347,7 +3392,7 @@
         <v>80</v>
       </c>
       <c r="Q2" s="22" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="R2" s="11" t="s">
         <v>80</v>
@@ -3368,19 +3413,19 @@
         <v>80</v>
       </c>
       <c r="X2" s="20" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="Y2" s="20" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="Z2" s="11" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="AA2" s="21" t="s">
-        <v>306</v>
-      </c>
-    </row>
-    <row r="3" spans="1:29" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="3" spans="1:29" ht="32.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="12" t="s">
         <v>70</v>
       </c>
@@ -3430,7 +3475,7 @@
         <v>80</v>
       </c>
       <c r="Q3" s="22" t="s">
-        <v>164</v>
+        <v>314</v>
       </c>
       <c r="R3" s="11" t="s">
         <v>80</v>
@@ -3451,24 +3496,24 @@
         <v>80</v>
       </c>
       <c r="X3" s="20" t="s">
-        <v>164</v>
+        <v>317</v>
       </c>
       <c r="Y3" s="20" t="s">
-        <v>164</v>
+        <v>320</v>
       </c>
       <c r="Z3" s="11" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="AA3" s="11" t="s">
-        <v>305</v>
-      </c>
-    </row>
-    <row r="4" spans="1:29" x14ac:dyDescent="0.3">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="4" spans="1:29" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="12" t="s">
         <v>69</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="C4" s="11" t="s">
         <v>80</v>
@@ -3477,7 +3522,7 @@
         <v>80</v>
       </c>
       <c r="E4" s="16" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="F4" s="11" t="s">
         <v>80</v>
@@ -3513,7 +3558,7 @@
         <v>80</v>
       </c>
       <c r="Q4" s="22" t="s">
-        <v>164</v>
+        <v>315</v>
       </c>
       <c r="R4" s="11" t="s">
         <v>80</v>
@@ -3534,10 +3579,10 @@
         <v>80</v>
       </c>
       <c r="X4" s="20" t="s">
-        <v>164</v>
+        <v>318</v>
       </c>
       <c r="Y4" s="20" t="s">
-        <v>164</v>
+        <v>321</v>
       </c>
       <c r="Z4" s="11" t="s">
         <v>80</v>
@@ -3546,7 +3591,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="5" spans="1:29" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:29" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="12" t="s">
         <v>71</v>
       </c>
@@ -3596,7 +3641,7 @@
         <v>80</v>
       </c>
       <c r="Q5" s="20" t="s">
-        <v>164</v>
+        <v>316</v>
       </c>
       <c r="R5" s="11" t="s">
         <v>80</v>
@@ -3617,10 +3662,10 @@
         <v>80</v>
       </c>
       <c r="X5" s="20" t="s">
-        <v>164</v>
+        <v>319</v>
       </c>
       <c r="Y5" s="20" t="s">
-        <v>164</v>
+        <v>322</v>
       </c>
       <c r="Z5" s="11" t="s">
         <v>80</v>
@@ -3637,79 +3682,79 @@
         <v>77</v>
       </c>
       <c r="C6" s="15" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="D6" s="15" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="E6" s="15" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="F6" s="15" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="G6" s="15" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="H6" s="15" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="I6" s="15" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="J6" s="15" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="K6" s="15" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="L6" s="15" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="M6" s="15" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="N6" s="15" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="O6" s="15" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="P6" s="15" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="Q6" s="20" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="R6" s="15" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="S6" s="15" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="T6" s="15" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="U6" s="15" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="V6" s="15" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="W6" s="15" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="X6" s="20" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="Y6" s="20" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="Z6" s="15" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="AA6" s="15" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
     </row>
     <row r="7" spans="1:29" ht="43.2" x14ac:dyDescent="0.3">
@@ -3720,79 +3765,79 @@
         <v>78</v>
       </c>
       <c r="C7" s="15" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="D7" s="15" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="E7" s="15" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="F7" s="15" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="G7" s="15" t="s">
         <v>81</v>
       </c>
       <c r="H7" s="15" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="I7" s="15" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="J7" s="15" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="K7" s="15" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="L7" s="15" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="M7" s="15" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="N7" s="15" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="O7" s="15" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="P7" s="15" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="Q7" s="20" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="R7" s="15" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="S7" s="15" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="T7" s="15" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="U7" s="15" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="V7" s="15" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="W7" s="15" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="X7" s="20" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="Y7" s="20" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="Z7" s="15" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="AA7" s="15" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
     </row>
     <row r="8" spans="1:29" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -3845,7 +3890,7 @@
         <v>82</v>
       </c>
       <c r="Q8" s="20" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="R8" s="4" t="s">
         <v>82</v>
@@ -3866,10 +3911,10 @@
         <v>82</v>
       </c>
       <c r="X8" s="20" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="Y8" s="20" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="Z8" s="4" t="s">
         <v>82</v>

</xml_diff>

<commit_message>
Updates to the speech files
</commit_message>
<xml_diff>
--- a/SpeechGenerationAudit.xlsx
+++ b/SpeechGenerationAudit.xlsx
@@ -8,16 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pc\Speech Generation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:2009_{D06D5749-81B6-44F1-BA47-2C9F1558BB54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F9B773E-92A3-4F93-92CD-713BC3CF5915}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="444" yWindow="3204" windowWidth="11808" windowHeight="9960" activeTab="1" xr2:uid="{A672C37D-E69E-470F-9024-46D64C3F6E80}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="13776" activeTab="1" xr2:uid="{A672C37D-E69E-470F-9024-46D64C3F6E80}"/>
   </bookViews>
   <sheets>
     <sheet name="Audio + String Table " sheetId="1" r:id="rId1"/>
     <sheet name="Only Audio" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -41,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="690" uniqueCount="323">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="690" uniqueCount="330">
   <si>
     <t>Unity Key</t>
   </si>
@@ -286,9 +285,6 @@
     <t xml:space="preserve">Accurate </t>
   </si>
   <si>
-    <t xml:space="preserve">Audio does not match (not only "Hat es Spass gemacht?", "Hast du Schmerzen gehabt?" as well) </t>
-  </si>
-  <si>
     <t>Need device to check</t>
   </si>
   <si>
@@ -532,9 +528,6 @@
     <t>Hebat! Kita boleh menikmati bersama!</t>
   </si>
   <si>
-    <t xml:space="preserve">No audio </t>
-  </si>
-  <si>
     <t>Unity Hausa Text</t>
   </si>
   <si>
@@ -964,18 +957,9 @@
     <t>Same meaning, different words</t>
   </si>
   <si>
-    <t xml:space="preserve">Audio matches the text under the heading (sort of) </t>
-  </si>
-  <si>
     <t xml:space="preserve">Audio matches filename, doesn't match r written (heading is just "Take a break", subheading is German speech prompt translated) </t>
   </si>
   <si>
-    <t xml:space="preserve">Audio does not match (same as German) </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Audio does not match (same as German)                                   </t>
-  </si>
-  <si>
     <t xml:space="preserve">Fixed </t>
   </si>
   <si>
@@ -985,31 +969,67 @@
     <t>No audio : FIXED</t>
   </si>
   <si>
-    <t xml:space="preserve">No audio: Buka kunci item yang dipilih? - FIXED </t>
-  </si>
-  <si>
-    <t>No audio : Awak nak berhenti kerja ke ? - FIXED</t>
-  </si>
-  <si>
-    <t>No audio: Anda tidak mempun yai syiling yang mencukupi - FIXED</t>
-  </si>
-  <si>
-    <t>No audio: தேர்ந்தெடுத்த பொருளை திறக்கவா? - FIXED</t>
-  </si>
-  <si>
-    <t>No audio: நீங்க வெளியேறணுமா? - FIXED</t>
-  </si>
-  <si>
-    <t>No audio: உங்களிடம் போதுமான நாணயங்கள் இல்லை. - FIXED</t>
-  </si>
-  <si>
-    <t>No audio: ปลดล็อกรายการที่เลือกใช่หรือไม่? - FIXED</t>
-  </si>
-  <si>
-    <t>No audio: คุณต้องการลาออกหรือไม่? - FIXED</t>
-  </si>
-  <si>
-    <t>No audio : คุณมีเหรียญไม่พอ - FIXED</t>
+    <t xml:space="preserve">No audio: Buka kunci item yang dipilih?  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">No audio : Awak nak berhenti kerja ke ? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">No audio: Anda tidak mempun yai syiling yang mencukupi </t>
+  </si>
+  <si>
+    <t xml:space="preserve">No audio: Adakah anda pasti tentang maklum balas itu? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">No audio: தேர்ந்தெடுத்த பொருளை திறக்கவா? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">No audio: நீங்க வெளியேறணுமா? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">No audio: உங்களிடம் போதுமான நாணயங்கள் இல்லை. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">No audio: ปลดล็อกรายการที่เลือกใช่หรือไม่? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">No audio : คุณมีเหรียญไม่พอ </t>
+  </si>
+  <si>
+    <t xml:space="preserve">No audio: คุณต้องการลาออกหรือไม่? </t>
+  </si>
+  <si>
+    <t>No audio: கருத்தை பற்றி உறுதியாக இருக்கிறீர்களா?</t>
+  </si>
+  <si>
+    <t>No audio: คุณแน่ใจเกี่ยวกับข้อเสนอแนะนั้นหรือเปล่า?</t>
+  </si>
+  <si>
+    <t>No audio : Anda sudah berlatih secukupnya, sila berehat sebentar sebelum meneruskan.</t>
+  </si>
+  <si>
+    <t>No audio : நீங்கள் போதுமான அளவு பயிற்சி செய்துள்ளீர்கள், தொடர்வதற்கு முன் ஒரு சிறிய இடைவேளை எடுத்துக் கொள்ளுங்கள்.</t>
+  </si>
+  <si>
+    <t>No audio : คุณฝึกมามากพอแล้ว โปรดพักสักครู่ก่อนฝึกต่อ</t>
+  </si>
+  <si>
+    <t>No audio: Sila kalibrasi pergerakan anda.</t>
+  </si>
+  <si>
+    <t>No audio: தயவுசெய்து உங்கள் இயக்கத்தை அளவீடு செய்யவும்.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No audio: โปรดปรับเทียบการเคลื่อนไหวของคุณ </t>
+  </si>
+  <si>
+    <t>No audio: Bagaimana perlawanan itu?</t>
+  </si>
+  <si>
+    <t>No audio: விளையாட்டு எப்படி இருந்தது?</t>
+  </si>
+  <si>
+    <t>No audio: เกมเป็นอย่างไรบ้าง?</t>
   </si>
 </sst>
 </file>
@@ -1575,25 +1595,25 @@
         <v>2</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>3</v>
@@ -1605,121 +1625,121 @@
         <v>3</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="N1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="P1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="R1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="T1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="V1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="X1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="Y1" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="Z1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="AA1" s="1" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="AB1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="AC1" s="1" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="AD1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="AE1" s="1" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="AF1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="AG1" s="1" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="AH1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="AI1" s="1" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="AJ1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="AK1" s="1" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="AL1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="AM1" s="1" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="AN1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="AO1" s="1" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="AP1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="AQ1" s="1" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="AR1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="AS1" s="1" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="AT1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="AU1" s="1" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="AV1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="AW1" s="1" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="AX1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="AY1" s="1" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="AZ1" s="1" t="s">
         <v>3</v>
@@ -1733,25 +1753,25 @@
         <v>63</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="D2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="F2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="G2" s="9" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="H2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="I2" s="9" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="J2" s="10" t="s">
         <v>56</v>
@@ -1763,121 +1783,121 @@
         <v>56</v>
       </c>
       <c r="M2" s="9" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="N2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="O2" s="9" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="P2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="Q2" s="9" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="R2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="S2" s="9" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="T2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="U2" s="9" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="V2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="W2" s="9" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="X2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="Y2" s="9" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="Z2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AA2" s="9" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="AB2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AC2" s="9" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="AD2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AE2" s="18" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="AF2" s="19" t="s">
-        <v>313</v>
+        <v>308</v>
       </c>
       <c r="AG2" s="9" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="AH2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AI2" s="9" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="AJ2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AK2" s="9" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="AL2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AM2" s="9" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="AN2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AO2" s="9" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="AP2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AQ2" s="9" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="AR2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AS2" s="18" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="AT2" s="19" t="s">
-        <v>313</v>
+        <v>308</v>
       </c>
       <c r="AU2" s="18" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="AV2" s="19" t="s">
-        <v>313</v>
+        <v>308</v>
       </c>
       <c r="AW2" s="9" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="AX2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AY2" s="9" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="AZ2" s="10" t="s">
         <v>56</v>
@@ -1891,25 +1911,25 @@
         <v>64</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="D3" s="10" t="s">
         <v>56</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="F3" s="10" t="s">
         <v>56</v>
       </c>
       <c r="G3" s="9" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="H3" s="10" t="s">
         <v>56</v>
       </c>
       <c r="I3" s="9" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="J3" s="10" t="s">
         <v>56</v>
@@ -1927,115 +1947,115 @@
         <v>56</v>
       </c>
       <c r="O3" s="9" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="P3" s="10" t="s">
         <v>56</v>
       </c>
       <c r="Q3" s="9" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="R3" s="10" t="s">
         <v>56</v>
       </c>
       <c r="S3" s="9" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="T3" s="10" t="s">
         <v>56</v>
       </c>
       <c r="U3" s="9" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="V3" s="10" t="s">
         <v>56</v>
       </c>
       <c r="W3" s="9" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="X3" s="10" t="s">
         <v>56</v>
       </c>
       <c r="Y3" s="9" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="Z3" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AA3" s="9" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="AB3" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AC3" s="9" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="AD3" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AE3" s="18" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="AF3" s="19" t="s">
-        <v>313</v>
+        <v>308</v>
       </c>
       <c r="AG3" s="9" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="AH3" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AI3" s="9" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="AJ3" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AK3" s="9" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="AL3" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AM3" s="9" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="AN3" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AO3" s="9" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="AP3" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AQ3" s="9" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="AR3" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AS3" s="18" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="AT3" s="19" t="s">
-        <v>313</v>
+        <v>308</v>
       </c>
       <c r="AU3" s="18" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="AV3" s="19" t="s">
-        <v>313</v>
+        <v>308</v>
       </c>
       <c r="AW3" s="9" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="AX3" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AY3" s="9" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="AZ3" s="10" t="s">
         <v>56</v>
@@ -2049,25 +2069,25 @@
         <v>60</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="D4" s="10" t="s">
         <v>56</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="F4" s="10" t="s">
         <v>56</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="H4" s="10" t="s">
         <v>56</v>
       </c>
       <c r="I4" s="9" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="J4" s="10" t="s">
         <v>56</v>
@@ -2079,121 +2099,121 @@
         <v>56</v>
       </c>
       <c r="M4" s="23" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="N4" s="24" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="O4" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="P4" s="10" t="s">
         <v>56</v>
       </c>
       <c r="Q4" s="16" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="R4" s="16" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="S4" s="9" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="T4" s="10" t="s">
         <v>56</v>
       </c>
       <c r="U4" s="9" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="V4" s="10" t="s">
         <v>56</v>
       </c>
       <c r="W4" s="9" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="X4" s="10" t="s">
         <v>56</v>
       </c>
       <c r="Y4" s="9" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="Z4" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AA4" s="9" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="AB4" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AC4" s="9" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="AD4" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AE4" s="18" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="AF4" s="19" t="s">
-        <v>313</v>
+        <v>308</v>
       </c>
       <c r="AG4" s="9" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="AH4" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AI4" s="9" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="AJ4" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AK4" s="9" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="AL4" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AM4" s="16" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="AN4" s="17" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="AO4" s="9" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="AP4" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AQ4" s="9" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="AR4" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AS4" s="18" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="AT4" s="19" t="s">
-        <v>313</v>
+        <v>308</v>
       </c>
       <c r="AU4" s="18" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="AV4" s="19" t="s">
-        <v>313</v>
+        <v>308</v>
       </c>
       <c r="AW4" s="9" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="AX4" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AY4" s="9" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="AZ4" s="10" t="s">
         <v>56</v>
@@ -2207,25 +2227,25 @@
         <v>57</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="D5" s="10" t="s">
         <v>56</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="F5" s="10" t="s">
         <v>56</v>
       </c>
       <c r="G5" s="9" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="H5" s="10" t="s">
         <v>56</v>
       </c>
       <c r="I5" s="9" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="J5" s="10" t="s">
         <v>56</v>
@@ -2237,121 +2257,121 @@
         <v>56</v>
       </c>
       <c r="M5" s="23" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="N5" s="24" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="O5" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="P5" s="10" t="s">
         <v>56</v>
       </c>
       <c r="Q5" s="9" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="R5" s="10" t="s">
         <v>56</v>
       </c>
       <c r="S5" s="9" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="T5" s="10" t="s">
         <v>56</v>
       </c>
       <c r="U5" s="9" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="V5" s="10" t="s">
         <v>56</v>
       </c>
       <c r="W5" s="9" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="X5" s="10" t="s">
         <v>56</v>
       </c>
       <c r="Y5" s="9" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Z5" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AA5" s="16" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="AB5" s="16" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="AC5" s="9" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="AD5" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AE5" s="18" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="AF5" s="19" t="s">
-        <v>313</v>
+        <v>308</v>
       </c>
       <c r="AG5" s="9" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="AH5" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AI5" s="9" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="AJ5" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AK5" s="9" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="AL5" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AM5" s="16" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="AN5" s="16" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="AO5" s="9" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="AP5" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AQ5" s="9" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="AR5" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AS5" s="18" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="AT5" s="19" t="s">
-        <v>313</v>
+        <v>308</v>
       </c>
       <c r="AU5" s="18" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="AV5" s="19" t="s">
-        <v>313</v>
+        <v>308</v>
       </c>
       <c r="AW5" s="9" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="AX5" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AY5" s="9" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="AZ5" s="10" t="s">
         <v>56</v>
@@ -2365,28 +2385,28 @@
         <v>58</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="D6" s="10" t="s">
         <v>59</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="F6" s="10" t="s">
         <v>59</v>
       </c>
       <c r="G6" s="9" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="H6" s="10" t="s">
         <v>59</v>
       </c>
       <c r="I6" s="9" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="J6" s="10" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="K6" s="9" t="s">
         <v>34</v>
@@ -2401,115 +2421,115 @@
         <v>59</v>
       </c>
       <c r="O6" s="9" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="P6" s="10" t="s">
         <v>59</v>
       </c>
       <c r="Q6" s="9" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="R6" s="10" t="s">
         <v>59</v>
       </c>
       <c r="S6" s="9" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="T6" s="10" t="s">
         <v>59</v>
       </c>
       <c r="U6" s="9" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="V6" s="10" t="s">
         <v>59</v>
       </c>
       <c r="W6" s="9" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="X6" s="10" t="s">
         <v>59</v>
       </c>
       <c r="Y6" s="9" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="Z6" s="10" t="s">
         <v>59</v>
       </c>
       <c r="AA6" s="16" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="AB6" s="16" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="AC6" s="9" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="AD6" s="10" t="s">
         <v>59</v>
       </c>
       <c r="AE6" s="18" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="AF6" s="19" t="s">
-        <v>313</v>
+        <v>308</v>
       </c>
       <c r="AG6" s="9" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="AH6" s="10" t="s">
         <v>59</v>
       </c>
       <c r="AI6" s="9" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="AJ6" s="10" t="s">
         <v>59</v>
       </c>
       <c r="AK6" s="9" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="AL6" s="10" t="s">
         <v>59</v>
       </c>
       <c r="AM6" s="9" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="AN6" s="10" t="s">
         <v>59</v>
       </c>
       <c r="AO6" s="9" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="AP6" s="10" t="s">
         <v>59</v>
       </c>
       <c r="AQ6" s="9" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="AR6" s="10" t="s">
         <v>59</v>
       </c>
       <c r="AS6" s="18" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="AT6" s="19" t="s">
-        <v>313</v>
+        <v>308</v>
       </c>
       <c r="AU6" s="18" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="AV6" s="19" t="s">
-        <v>313</v>
+        <v>308</v>
       </c>
       <c r="AW6" s="9" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="AX6" s="10" t="s">
         <v>59</v>
       </c>
       <c r="AY6" s="9" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="AZ6" s="10" t="s">
         <v>59</v>
@@ -2523,25 +2543,25 @@
         <v>61</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="D7" s="10" t="s">
         <v>56</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="F7" s="10" t="s">
         <v>56</v>
       </c>
       <c r="G7" s="9" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="H7" s="10" t="s">
         <v>56</v>
       </c>
       <c r="I7" s="9" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="J7" s="10" t="s">
         <v>56</v>
@@ -2553,121 +2573,121 @@
         <v>56</v>
       </c>
       <c r="M7" s="9" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="N7" s="10" t="s">
         <v>56</v>
       </c>
       <c r="O7" s="9" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="P7" s="10" t="s">
         <v>56</v>
       </c>
       <c r="Q7" s="16" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="R7" s="16" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="S7" s="9" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="T7" s="10" t="s">
         <v>56</v>
       </c>
       <c r="U7" s="9" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="V7" s="10" t="s">
         <v>56</v>
       </c>
       <c r="W7" s="9" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="X7" s="10" t="s">
         <v>56</v>
       </c>
       <c r="Y7" s="9" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="Z7" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AA7" s="16" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="AB7" s="16" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="AC7" s="9" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="AD7" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AE7" s="18" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="AF7" s="19" t="s">
-        <v>313</v>
+        <v>308</v>
       </c>
       <c r="AG7" s="9" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="AH7" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AI7" s="9" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="AJ7" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AK7" s="9" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="AL7" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AM7" s="16" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="AN7" s="17" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="AO7" s="9" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="AP7" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AQ7" s="9" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="AR7" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AS7" s="18" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="AT7" s="19" t="s">
-        <v>313</v>
+        <v>308</v>
       </c>
       <c r="AU7" s="18" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="AV7" s="19" t="s">
-        <v>313</v>
+        <v>308</v>
       </c>
       <c r="AW7" s="9" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="AX7" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AY7" s="9" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="AZ7" s="10" t="s">
         <v>56</v>
@@ -2681,25 +2701,25 @@
         <v>62</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="D8" s="10" t="s">
         <v>56</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="F8" s="10" t="s">
         <v>56</v>
       </c>
       <c r="G8" s="9" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="H8" s="10" t="s">
         <v>56</v>
       </c>
       <c r="I8" s="9" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="J8" s="10" t="s">
         <v>56</v>
@@ -2717,115 +2737,115 @@
         <v>56</v>
       </c>
       <c r="O8" s="9" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="P8" s="10" t="s">
         <v>56</v>
       </c>
       <c r="Q8" s="9" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="R8" s="10" t="s">
         <v>56</v>
       </c>
       <c r="S8" s="9" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="T8" s="10" t="s">
         <v>56</v>
       </c>
       <c r="U8" s="9" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="V8" s="10" t="s">
         <v>56</v>
       </c>
       <c r="W8" s="9" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="X8" s="10" t="s">
         <v>56</v>
       </c>
       <c r="Y8" s="9" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="Z8" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AA8" s="9" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="AB8" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AC8" s="9" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="AD8" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AE8" s="18" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="AF8" s="19" t="s">
-        <v>313</v>
+        <v>308</v>
       </c>
       <c r="AG8" s="9" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="AH8" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AI8" s="9" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="AJ8" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AK8" s="9" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="AL8" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AM8" s="9" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="AN8" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AO8" s="9" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="AP8" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AQ8" s="9" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="AR8" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AS8" s="18" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="AT8" s="19" t="s">
-        <v>313</v>
+        <v>308</v>
       </c>
       <c r="AU8" s="18" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="AV8" s="19" t="s">
-        <v>313</v>
+        <v>308</v>
       </c>
       <c r="AW8" s="9" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="AX8" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AY8" s="9" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="AZ8" s="10" t="s">
         <v>56</v>
@@ -2888,7 +2908,7 @@
         <v>39</v>
       </c>
       <c r="AL11" s="19" t="s">
-        <v>312</v>
+        <v>307</v>
       </c>
     </row>
     <row r="12" spans="1:52" x14ac:dyDescent="0.3">
@@ -3244,7 +3264,7 @@
     <col min="14" max="14" width="26.44140625" customWidth="1"/>
     <col min="15" max="15" width="28.5546875" customWidth="1"/>
     <col min="16" max="16" width="26.33203125" customWidth="1"/>
-    <col min="17" max="17" width="38.88671875" customWidth="1"/>
+    <col min="17" max="17" width="46.21875" customWidth="1"/>
     <col min="18" max="18" width="27.109375" customWidth="1"/>
     <col min="19" max="19" width="26.6640625" customWidth="1"/>
     <col min="20" max="20" width="31.33203125" customWidth="1"/>
@@ -3265,84 +3285,84 @@
         <v>67</v>
       </c>
       <c r="C1" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>278</v>
+      </c>
+      <c r="E1" s="6" t="s">
         <v>279</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="F1" s="6" t="s">
         <v>280</v>
-      </c>
-      <c r="E1" s="6" t="s">
-        <v>281</v>
-      </c>
-      <c r="F1" s="6" t="s">
-        <v>282</v>
       </c>
       <c r="G1" s="6" t="s">
         <v>68</v>
       </c>
       <c r="H1" s="6" t="s">
+        <v>281</v>
+      </c>
+      <c r="I1" s="6" t="s">
+        <v>282</v>
+      </c>
+      <c r="J1" s="6" t="s">
         <v>283</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="K1" s="6" t="s">
         <v>284</v>
       </c>
-      <c r="J1" s="6" t="s">
+      <c r="L1" s="6" t="s">
         <v>285</v>
       </c>
-      <c r="K1" s="6" t="s">
+      <c r="M1" s="6" t="s">
         <v>286</v>
       </c>
-      <c r="L1" s="6" t="s">
+      <c r="N1" s="6" t="s">
         <v>287</v>
       </c>
-      <c r="M1" s="6" t="s">
+      <c r="O1" s="6" t="s">
         <v>288</v>
       </c>
-      <c r="N1" s="6" t="s">
+      <c r="P1" s="6" t="s">
         <v>289</v>
       </c>
-      <c r="O1" s="6" t="s">
+      <c r="Q1" s="6" t="s">
         <v>290</v>
       </c>
-      <c r="P1" s="6" t="s">
+      <c r="R1" s="6" t="s">
         <v>291</v>
       </c>
-      <c r="Q1" s="6" t="s">
+      <c r="S1" s="6" t="s">
         <v>292</v>
       </c>
-      <c r="R1" s="6" t="s">
+      <c r="T1" s="6" t="s">
         <v>293</v>
       </c>
-      <c r="S1" s="6" t="s">
+      <c r="U1" s="6" t="s">
         <v>294</v>
       </c>
-      <c r="T1" s="6" t="s">
+      <c r="V1" s="6" t="s">
         <v>295</v>
       </c>
-      <c r="U1" s="6" t="s">
+      <c r="W1" s="6" t="s">
         <v>296</v>
       </c>
-      <c r="V1" s="6" t="s">
+      <c r="X1" s="6" t="s">
         <v>297</v>
       </c>
-      <c r="W1" s="6" t="s">
+      <c r="Y1" s="6" t="s">
         <v>298</v>
       </c>
-      <c r="X1" s="6" t="s">
+      <c r="Z1" s="6" t="s">
         <v>299</v>
       </c>
-      <c r="Y1" s="6" t="s">
+      <c r="AA1" s="6" t="s">
         <v>300</v>
-      </c>
-      <c r="Z1" s="6" t="s">
-        <v>301</v>
-      </c>
-      <c r="AA1" s="6" t="s">
-        <v>302</v>
       </c>
       <c r="AB1" s="6"/>
       <c r="AC1" s="6"/>
     </row>
-    <row r="2" spans="1:29" ht="21" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:29" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="11">
         <v>3</v>
       </c>
@@ -3392,7 +3412,7 @@
         <v>80</v>
       </c>
       <c r="Q2" s="22" t="s">
-        <v>163</v>
+        <v>312</v>
       </c>
       <c r="R2" s="11" t="s">
         <v>80</v>
@@ -3413,16 +3433,16 @@
         <v>80</v>
       </c>
       <c r="X2" s="20" t="s">
-        <v>163</v>
+        <v>319</v>
       </c>
       <c r="Y2" s="20" t="s">
-        <v>163</v>
+        <v>320</v>
       </c>
       <c r="Z2" s="11" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="AA2" s="21" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
     </row>
     <row r="3" spans="1:29" ht="32.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -3475,7 +3495,7 @@
         <v>80</v>
       </c>
       <c r="Q3" s="22" t="s">
-        <v>314</v>
+        <v>309</v>
       </c>
       <c r="R3" s="11" t="s">
         <v>80</v>
@@ -3496,16 +3516,16 @@
         <v>80</v>
       </c>
       <c r="X3" s="20" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
       <c r="Y3" s="20" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
       <c r="Z3" s="11" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="AA3" s="11" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
     </row>
     <row r="4" spans="1:29" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -3513,7 +3533,7 @@
         <v>69</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="C4" s="11" t="s">
         <v>80</v>
@@ -3522,7 +3542,7 @@
         <v>80</v>
       </c>
       <c r="E4" s="16" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="F4" s="11" t="s">
         <v>80</v>
@@ -3558,7 +3578,7 @@
         <v>80</v>
       </c>
       <c r="Q4" s="22" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="R4" s="11" t="s">
         <v>80</v>
@@ -3579,10 +3599,10 @@
         <v>80</v>
       </c>
       <c r="X4" s="20" t="s">
+        <v>314</v>
+      </c>
+      <c r="Y4" s="20" t="s">
         <v>318</v>
-      </c>
-      <c r="Y4" s="20" t="s">
-        <v>321</v>
       </c>
       <c r="Z4" s="11" t="s">
         <v>80</v>
@@ -3641,7 +3661,7 @@
         <v>80</v>
       </c>
       <c r="Q5" s="20" t="s">
-        <v>316</v>
+        <v>311</v>
       </c>
       <c r="R5" s="11" t="s">
         <v>80</v>
@@ -3662,10 +3682,10 @@
         <v>80</v>
       </c>
       <c r="X5" s="20" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="Y5" s="20" t="s">
-        <v>322</v>
+        <v>317</v>
       </c>
       <c r="Z5" s="11" t="s">
         <v>80</v>
@@ -3682,162 +3702,162 @@
         <v>77</v>
       </c>
       <c r="C6" s="15" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="D6" s="15" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="E6" s="15" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="F6" s="15" t="s">
-        <v>308</v>
-      </c>
-      <c r="G6" s="15" t="s">
-        <v>307</v>
+        <v>305</v>
+      </c>
+      <c r="G6" s="11" t="s">
+        <v>80</v>
       </c>
       <c r="H6" s="15" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="I6" s="15" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="J6" s="15" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K6" s="15" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="L6" s="15" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="M6" s="15" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="N6" s="15" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="O6" s="15" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="P6" s="15" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="Q6" s="20" t="s">
-        <v>163</v>
+        <v>321</v>
       </c>
       <c r="R6" s="15" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="S6" s="15" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="T6" s="15" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="U6" s="15" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="V6" s="15" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="W6" s="15" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="X6" s="20" t="s">
-        <v>163</v>
+        <v>322</v>
       </c>
       <c r="Y6" s="20" t="s">
-        <v>163</v>
+        <v>323</v>
       </c>
       <c r="Z6" s="15" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="AA6" s="15" t="s">
-        <v>308</v>
-      </c>
-    </row>
-    <row r="7" spans="1:29" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A7" s="13" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="7" spans="1:29" x14ac:dyDescent="0.3">
+      <c r="A7" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="B7" s="14" t="s">
+      <c r="B7" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="C7" s="15" t="s">
-        <v>309</v>
-      </c>
-      <c r="D7" s="15" t="s">
-        <v>310</v>
-      </c>
-      <c r="E7" s="15" t="s">
-        <v>309</v>
-      </c>
-      <c r="F7" s="15" t="s">
-        <v>309</v>
-      </c>
-      <c r="G7" s="15" t="s">
-        <v>81</v>
-      </c>
-      <c r="H7" s="15" t="s">
-        <v>309</v>
-      </c>
-      <c r="I7" s="15" t="s">
-        <v>309</v>
-      </c>
-      <c r="J7" s="15" t="s">
-        <v>309</v>
-      </c>
-      <c r="K7" s="15" t="s">
-        <v>309</v>
-      </c>
-      <c r="L7" s="15" t="s">
-        <v>309</v>
-      </c>
-      <c r="M7" s="15" t="s">
-        <v>309</v>
-      </c>
-      <c r="N7" s="15" t="s">
-        <v>309</v>
-      </c>
-      <c r="O7" s="15" t="s">
-        <v>309</v>
-      </c>
-      <c r="P7" s="15" t="s">
-        <v>309</v>
+      <c r="C7" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="D7" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="E7" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="F7" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="G7" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="H7" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="I7" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="J7" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="K7" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="L7" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="M7" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="N7" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="O7" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="P7" s="11" t="s">
+        <v>80</v>
       </c>
       <c r="Q7" s="20" t="s">
-        <v>163</v>
-      </c>
-      <c r="R7" s="15" t="s">
-        <v>309</v>
-      </c>
-      <c r="S7" s="15" t="s">
-        <v>309</v>
-      </c>
-      <c r="T7" s="15" t="s">
-        <v>309</v>
-      </c>
-      <c r="U7" s="15" t="s">
-        <v>309</v>
-      </c>
-      <c r="V7" s="15" t="s">
-        <v>309</v>
-      </c>
-      <c r="W7" s="15" t="s">
-        <v>309</v>
+        <v>327</v>
+      </c>
+      <c r="R7" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="S7" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="T7" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="U7" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="V7" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="W7" s="11" t="s">
+        <v>80</v>
       </c>
       <c r="X7" s="20" t="s">
-        <v>163</v>
+        <v>328</v>
       </c>
       <c r="Y7" s="20" t="s">
-        <v>163</v>
-      </c>
-      <c r="Z7" s="15" t="s">
-        <v>309</v>
-      </c>
-      <c r="AA7" s="15" t="s">
-        <v>309</v>
+        <v>329</v>
+      </c>
+      <c r="Z7" s="11" t="s">
+        <v>301</v>
+      </c>
+      <c r="AA7" s="11" t="s">
+        <v>301</v>
       </c>
     </row>
     <row r="8" spans="1:29" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -3848,79 +3868,79 @@
         <v>79</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="I8" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J8" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="K8" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="L8" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="M8" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="N8" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="O8" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="P8" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="Q8" s="20" t="s">
-        <v>163</v>
+        <v>324</v>
       </c>
       <c r="R8" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="S8" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="T8" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="U8" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="V8" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="W8" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="X8" s="20" t="s">
-        <v>163</v>
+        <v>325</v>
       </c>
       <c r="Y8" s="20" t="s">
-        <v>163</v>
+        <v>326</v>
       </c>
       <c r="Z8" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AA8" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="9" spans="1:29" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Additional speech files generated, table extension
</commit_message>
<xml_diff>
--- a/SpeechGenerationAudit.xlsx
+++ b/SpeechGenerationAudit.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pc\Speech Generation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F9B773E-92A3-4F93-92CD-713BC3CF5915}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA6D698E-4A88-405C-A4C2-895588681F36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="13776" activeTab="1" xr2:uid="{A672C37D-E69E-470F-9024-46D64C3F6E80}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{A672C37D-E69E-470F-9024-46D64C3F6E80}"/>
   </bookViews>
   <sheets>
     <sheet name="Audio + String Table " sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="690" uniqueCount="330">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="717" uniqueCount="335">
   <si>
     <t>Unity Key</t>
   </si>
@@ -267,9 +267,6 @@
     <t>Calibrate</t>
   </si>
   <si>
-    <t>Unlock the game</t>
-  </si>
-  <si>
     <t>You don_t have enough coins</t>
   </si>
   <si>
@@ -1030,6 +1027,24 @@
   </si>
   <si>
     <t>No audio: เกมเป็นอย่างไรบ้าง?</t>
+  </si>
+  <si>
+    <t>UnlockSelectedItem</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unlock the selected item </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unlock the game </t>
+  </si>
+  <si>
+    <t>No audio: Buka kunci permainan ini?</t>
+  </si>
+  <si>
+    <t>No audio: விளையாட்டை திறக்கவா?</t>
+  </si>
+  <si>
+    <t>No audio: ปลดล็อกเกมใช่หรือไม่?</t>
   </si>
 </sst>
 </file>
@@ -1595,25 +1610,25 @@
         <v>2</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>3</v>
@@ -1625,121 +1640,121 @@
         <v>3</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="N1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="P1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="R1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="T1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="V1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="X1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="Y1" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Z1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="AA1" s="1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="AB1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="AC1" s="1" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="AD1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="AE1" s="1" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="AF1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="AG1" s="1" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="AH1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="AI1" s="1" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="AJ1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="AK1" s="1" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="AL1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="AM1" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="AN1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="AO1" s="1" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="AP1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="AQ1" s="1" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="AR1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="AS1" s="1" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="AT1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="AU1" s="1" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="AV1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="AW1" s="1" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="AX1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="AY1" s="1" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="AZ1" s="1" t="s">
         <v>3</v>
@@ -1753,25 +1768,25 @@
         <v>63</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="D2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="E2" s="9" t="s">
+        <v>254</v>
+      </c>
+      <c r="F2" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="G2" s="9" t="s">
         <v>255</v>
       </c>
-      <c r="F2" s="10" t="s">
-        <v>56</v>
-      </c>
-      <c r="G2" s="9" t="s">
-        <v>256</v>
-      </c>
       <c r="H2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="I2" s="9" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="J2" s="10" t="s">
         <v>56</v>
@@ -1783,121 +1798,121 @@
         <v>56</v>
       </c>
       <c r="M2" s="9" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="N2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="O2" s="9" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="P2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="Q2" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="R2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="S2" s="9" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="T2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="U2" s="9" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="V2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="W2" s="9" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="X2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="Y2" s="9" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="Z2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AA2" s="9" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="AB2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AC2" s="9" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="AD2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AE2" s="18" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="AF2" s="19" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="AG2" s="9" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="AH2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AI2" s="9" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="AJ2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AK2" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="AL2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AM2" s="9" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="AN2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AO2" s="9" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="AP2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AQ2" s="9" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="AR2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AS2" s="18" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="AT2" s="19" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="AU2" s="18" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="AV2" s="19" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="AW2" s="9" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AX2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AY2" s="9" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="AZ2" s="10" t="s">
         <v>56</v>
@@ -1911,25 +1926,25 @@
         <v>64</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="D3" s="10" t="s">
         <v>56</v>
       </c>
       <c r="E3" s="9" t="s">
+        <v>256</v>
+      </c>
+      <c r="F3" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="G3" s="9" t="s">
         <v>257</v>
       </c>
-      <c r="F3" s="10" t="s">
-        <v>56</v>
-      </c>
-      <c r="G3" s="9" t="s">
-        <v>258</v>
-      </c>
       <c r="H3" s="10" t="s">
         <v>56</v>
       </c>
       <c r="I3" s="9" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="J3" s="10" t="s">
         <v>56</v>
@@ -1947,115 +1962,115 @@
         <v>56</v>
       </c>
       <c r="O3" s="9" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="P3" s="10" t="s">
         <v>56</v>
       </c>
       <c r="Q3" s="9" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="R3" s="10" t="s">
         <v>56</v>
       </c>
       <c r="S3" s="9" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="T3" s="10" t="s">
         <v>56</v>
       </c>
       <c r="U3" s="9" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="V3" s="10" t="s">
         <v>56</v>
       </c>
       <c r="W3" s="9" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="X3" s="10" t="s">
         <v>56</v>
       </c>
       <c r="Y3" s="9" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="Z3" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AA3" s="9" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="AB3" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AC3" s="9" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="AD3" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AE3" s="18" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="AF3" s="19" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="AG3" s="9" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="AH3" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AI3" s="9" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="AJ3" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AK3" s="9" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="AL3" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AM3" s="9" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="AN3" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AO3" s="9" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="AP3" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AQ3" s="9" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="AR3" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AS3" s="18" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="AT3" s="19" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="AU3" s="18" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="AV3" s="19" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="AW3" s="9" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="AX3" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AY3" s="9" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="AZ3" s="10" t="s">
         <v>56</v>
@@ -2069,25 +2084,25 @@
         <v>60</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="D4" s="10" t="s">
         <v>56</v>
       </c>
       <c r="E4" s="9" t="s">
+        <v>258</v>
+      </c>
+      <c r="F4" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="G4" s="9" t="s">
         <v>259</v>
       </c>
-      <c r="F4" s="10" t="s">
-        <v>56</v>
-      </c>
-      <c r="G4" s="9" t="s">
-        <v>260</v>
-      </c>
       <c r="H4" s="10" t="s">
         <v>56</v>
       </c>
       <c r="I4" s="9" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="J4" s="10" t="s">
         <v>56</v>
@@ -2099,121 +2114,121 @@
         <v>56</v>
       </c>
       <c r="M4" s="23" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="N4" s="24" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="O4" s="9" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="P4" s="10" t="s">
         <v>56</v>
       </c>
       <c r="Q4" s="16" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="R4" s="16" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="S4" s="9" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="T4" s="10" t="s">
         <v>56</v>
       </c>
       <c r="U4" s="9" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="V4" s="10" t="s">
         <v>56</v>
       </c>
       <c r="W4" s="9" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="X4" s="10" t="s">
         <v>56</v>
       </c>
       <c r="Y4" s="9" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="Z4" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AA4" s="9" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="AB4" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AC4" s="9" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="AD4" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AE4" s="18" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="AF4" s="19" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="AG4" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="AH4" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AI4" s="9" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="AJ4" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AK4" s="9" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="AL4" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AM4" s="16" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="AN4" s="17" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="AO4" s="9" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="AP4" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AQ4" s="9" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="AR4" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AS4" s="18" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="AT4" s="19" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="AU4" s="18" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="AV4" s="19" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="AW4" s="9" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="AX4" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AY4" s="9" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="AZ4" s="10" t="s">
         <v>56</v>
@@ -2227,25 +2242,25 @@
         <v>57</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="D5" s="10" t="s">
         <v>56</v>
       </c>
       <c r="E5" s="9" t="s">
+        <v>260</v>
+      </c>
+      <c r="F5" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="G5" s="9" t="s">
         <v>261</v>
       </c>
-      <c r="F5" s="10" t="s">
-        <v>56</v>
-      </c>
-      <c r="G5" s="9" t="s">
-        <v>262</v>
-      </c>
       <c r="H5" s="10" t="s">
         <v>56</v>
       </c>
       <c r="I5" s="9" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="J5" s="10" t="s">
         <v>56</v>
@@ -2257,121 +2272,121 @@
         <v>56</v>
       </c>
       <c r="M5" s="23" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="N5" s="24" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="O5" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="P5" s="10" t="s">
         <v>56</v>
       </c>
       <c r="Q5" s="9" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="R5" s="10" t="s">
         <v>56</v>
       </c>
       <c r="S5" s="9" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="T5" s="10" t="s">
         <v>56</v>
       </c>
       <c r="U5" s="9" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="V5" s="10" t="s">
         <v>56</v>
       </c>
       <c r="W5" s="9" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="X5" s="10" t="s">
         <v>56</v>
       </c>
       <c r="Y5" s="9" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="Z5" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AA5" s="16" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="AB5" s="16" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="AC5" s="9" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="AD5" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AE5" s="18" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="AF5" s="19" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="AG5" s="9" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="AH5" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AI5" s="9" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="AJ5" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AK5" s="9" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="AL5" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AM5" s="16" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="AN5" s="16" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="AO5" s="9" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="AP5" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AQ5" s="9" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AR5" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AS5" s="18" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="AT5" s="19" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="AU5" s="18" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="AV5" s="19" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="AW5" s="9" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="AX5" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AY5" s="9" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="AZ5" s="10" t="s">
         <v>56</v>
@@ -2385,28 +2400,28 @@
         <v>58</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="D6" s="10" t="s">
         <v>59</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="F6" s="10" t="s">
         <v>59</v>
       </c>
       <c r="G6" s="9" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="H6" s="10" t="s">
         <v>59</v>
       </c>
       <c r="I6" s="9" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="J6" s="10" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="K6" s="9" t="s">
         <v>34</v>
@@ -2421,115 +2436,115 @@
         <v>59</v>
       </c>
       <c r="O6" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="P6" s="10" t="s">
         <v>59</v>
       </c>
       <c r="Q6" s="9" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="R6" s="10" t="s">
         <v>59</v>
       </c>
       <c r="S6" s="9" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="T6" s="10" t="s">
         <v>59</v>
       </c>
       <c r="U6" s="9" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="V6" s="10" t="s">
         <v>59</v>
       </c>
       <c r="W6" s="9" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="X6" s="10" t="s">
         <v>59</v>
       </c>
       <c r="Y6" s="9" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Z6" s="10" t="s">
         <v>59</v>
       </c>
       <c r="AA6" s="16" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="AB6" s="16" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="AC6" s="9" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="AD6" s="10" t="s">
         <v>59</v>
       </c>
       <c r="AE6" s="18" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="AF6" s="19" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="AG6" s="9" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="AH6" s="10" t="s">
         <v>59</v>
       </c>
       <c r="AI6" s="9" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="AJ6" s="10" t="s">
         <v>59</v>
       </c>
       <c r="AK6" s="9" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AL6" s="10" t="s">
         <v>59</v>
       </c>
       <c r="AM6" s="9" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="AN6" s="10" t="s">
         <v>59</v>
       </c>
       <c r="AO6" s="9" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="AP6" s="10" t="s">
         <v>59</v>
       </c>
       <c r="AQ6" s="9" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="AR6" s="10" t="s">
         <v>59</v>
       </c>
       <c r="AS6" s="18" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="AT6" s="19" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="AU6" s="18" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="AV6" s="19" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="AW6" s="9" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="AX6" s="10" t="s">
         <v>59</v>
       </c>
       <c r="AY6" s="9" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="AZ6" s="10" t="s">
         <v>59</v>
@@ -2543,25 +2558,25 @@
         <v>61</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="D7" s="10" t="s">
         <v>56</v>
       </c>
       <c r="E7" s="9" t="s">
+        <v>264</v>
+      </c>
+      <c r="F7" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="G7" s="9" t="s">
         <v>265</v>
       </c>
-      <c r="F7" s="10" t="s">
-        <v>56</v>
-      </c>
-      <c r="G7" s="9" t="s">
-        <v>266</v>
-      </c>
       <c r="H7" s="10" t="s">
         <v>56</v>
       </c>
       <c r="I7" s="9" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="J7" s="10" t="s">
         <v>56</v>
@@ -2573,121 +2588,121 @@
         <v>56</v>
       </c>
       <c r="M7" s="9" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="N7" s="10" t="s">
         <v>56</v>
       </c>
       <c r="O7" s="9" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="P7" s="10" t="s">
         <v>56</v>
       </c>
       <c r="Q7" s="16" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="R7" s="16" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="S7" s="9" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="T7" s="10" t="s">
         <v>56</v>
       </c>
       <c r="U7" s="9" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="V7" s="10" t="s">
         <v>56</v>
       </c>
       <c r="W7" s="9" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="X7" s="10" t="s">
         <v>56</v>
       </c>
       <c r="Y7" s="9" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="Z7" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AA7" s="16" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="AB7" s="16" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="AC7" s="9" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="AD7" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AE7" s="18" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="AF7" s="19" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="AG7" s="9" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="AH7" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AI7" s="9" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="AJ7" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AK7" s="9" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="AL7" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AM7" s="16" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="AN7" s="17" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="AO7" s="9" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="AP7" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AQ7" s="9" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="AR7" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AS7" s="18" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="AT7" s="19" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="AU7" s="18" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="AV7" s="19" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="AW7" s="9" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="AX7" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AY7" s="9" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="AZ7" s="10" t="s">
         <v>56</v>
@@ -2701,25 +2716,25 @@
         <v>62</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="D8" s="10" t="s">
         <v>56</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="F8" s="10" t="s">
         <v>56</v>
       </c>
       <c r="G8" s="9" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="H8" s="10" t="s">
         <v>56</v>
       </c>
       <c r="I8" s="9" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="J8" s="10" t="s">
         <v>56</v>
@@ -2737,115 +2752,115 @@
         <v>56</v>
       </c>
       <c r="O8" s="9" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="P8" s="10" t="s">
         <v>56</v>
       </c>
       <c r="Q8" s="9" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="R8" s="10" t="s">
         <v>56</v>
       </c>
       <c r="S8" s="9" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="T8" s="10" t="s">
         <v>56</v>
       </c>
       <c r="U8" s="9" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="V8" s="10" t="s">
         <v>56</v>
       </c>
       <c r="W8" s="9" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="X8" s="10" t="s">
         <v>56</v>
       </c>
       <c r="Y8" s="9" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="Z8" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AA8" s="9" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="AB8" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AC8" s="9" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="AD8" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AE8" s="18" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="AF8" s="19" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="AG8" s="9" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="AH8" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AI8" s="9" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="AJ8" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AK8" s="9" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="AL8" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AM8" s="9" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="AN8" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AO8" s="9" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="AP8" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AQ8" s="9" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="AR8" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AS8" s="18" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="AT8" s="19" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="AU8" s="18" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="AV8" s="19" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="AW8" s="9" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="AX8" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AY8" s="9" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AZ8" s="10" t="s">
         <v>56</v>
@@ -2908,7 +2923,7 @@
         <v>39</v>
       </c>
       <c r="AL11" s="19" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="12" spans="1:52" x14ac:dyDescent="0.3">
@@ -3245,10 +3260,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF649BE3-FEAC-4104-AA1F-4B0062E39075}">
-  <dimension ref="A1:AC30"/>
+  <dimension ref="A1:AC31"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.6640625" customWidth="1"/>
+    <col min="1" max="1" width="20.33203125" customWidth="1"/>
     <col min="2" max="2" width="28.5546875" customWidth="1"/>
     <col min="3" max="3" width="26.5546875" customWidth="1"/>
     <col min="4" max="4" width="29" customWidth="1"/>
@@ -3285,79 +3300,79 @@
         <v>67</v>
       </c>
       <c r="C1" s="6" t="s">
+        <v>276</v>
+      </c>
+      <c r="D1" s="6" t="s">
         <v>277</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="E1" s="6" t="s">
         <v>278</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="F1" s="6" t="s">
         <v>279</v>
-      </c>
-      <c r="F1" s="6" t="s">
-        <v>280</v>
       </c>
       <c r="G1" s="6" t="s">
         <v>68</v>
       </c>
       <c r="H1" s="6" t="s">
+        <v>280</v>
+      </c>
+      <c r="I1" s="6" t="s">
         <v>281</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="J1" s="6" t="s">
         <v>282</v>
       </c>
-      <c r="J1" s="6" t="s">
+      <c r="K1" s="6" t="s">
         <v>283</v>
       </c>
-      <c r="K1" s="6" t="s">
+      <c r="L1" s="6" t="s">
         <v>284</v>
       </c>
-      <c r="L1" s="6" t="s">
+      <c r="M1" s="6" t="s">
         <v>285</v>
       </c>
-      <c r="M1" s="6" t="s">
+      <c r="N1" s="6" t="s">
         <v>286</v>
       </c>
-      <c r="N1" s="6" t="s">
+      <c r="O1" s="6" t="s">
         <v>287</v>
       </c>
-      <c r="O1" s="6" t="s">
+      <c r="P1" s="6" t="s">
         <v>288</v>
       </c>
-      <c r="P1" s="6" t="s">
+      <c r="Q1" s="6" t="s">
         <v>289</v>
       </c>
-      <c r="Q1" s="6" t="s">
+      <c r="R1" s="6" t="s">
         <v>290</v>
       </c>
-      <c r="R1" s="6" t="s">
+      <c r="S1" s="6" t="s">
         <v>291</v>
       </c>
-      <c r="S1" s="6" t="s">
+      <c r="T1" s="6" t="s">
         <v>292</v>
       </c>
-      <c r="T1" s="6" t="s">
+      <c r="U1" s="6" t="s">
         <v>293</v>
       </c>
-      <c r="U1" s="6" t="s">
+      <c r="V1" s="6" t="s">
         <v>294</v>
       </c>
-      <c r="V1" s="6" t="s">
+      <c r="W1" s="6" t="s">
         <v>295</v>
       </c>
-      <c r="W1" s="6" t="s">
+      <c r="X1" s="6" t="s">
         <v>296</v>
       </c>
-      <c r="X1" s="6" t="s">
+      <c r="Y1" s="6" t="s">
         <v>297</v>
       </c>
-      <c r="Y1" s="6" t="s">
+      <c r="Z1" s="6" t="s">
         <v>298</v>
       </c>
-      <c r="Z1" s="6" t="s">
+      <c r="AA1" s="6" t="s">
         <v>299</v>
-      </c>
-      <c r="AA1" s="6" t="s">
-        <v>300</v>
       </c>
       <c r="AB1" s="6"/>
       <c r="AC1" s="6"/>
@@ -3370,593 +3385,661 @@
         <v>65</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E2" s="11" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F2" s="11" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="G2" s="11" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H2" s="11" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I2" s="11" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J2" s="11" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="K2" s="11" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="L2" s="11" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="M2" s="11" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="N2" s="11" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="O2" s="11" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="P2" s="11" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="Q2" s="22" t="s">
+        <v>311</v>
+      </c>
+      <c r="R2" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="S2" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="T2" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="U2" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="V2" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="W2" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="X2" s="20" t="s">
+        <v>318</v>
+      </c>
+      <c r="Y2" s="20" t="s">
+        <v>319</v>
+      </c>
+      <c r="Z2" s="11" t="s">
+        <v>300</v>
+      </c>
+      <c r="AA2" s="21" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="3" spans="1:29" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="11" t="s">
+        <v>70</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>331</v>
+      </c>
+      <c r="C3" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="D3" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="E3" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="F3" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="G3" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="H3" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="I3" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="J3" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="K3" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="L3" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="M3" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="N3" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="O3" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="P3" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="Q3" s="22" t="s">
+        <v>332</v>
+      </c>
+      <c r="R3" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="S3" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="T3" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="U3" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="V3" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="W3" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="X3" s="20" t="s">
+        <v>333</v>
+      </c>
+      <c r="Y3" s="20" t="s">
+        <v>334</v>
+      </c>
+      <c r="Z3" s="11" t="s">
+        <v>300</v>
+      </c>
+      <c r="AA3" s="11" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="4" spans="1:29" ht="32.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="12" t="s">
+        <v>329</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>330</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="D4" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="E4" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="F4" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="G4" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="H4" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="I4" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="J4" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="K4" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="L4" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="M4" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="N4" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="O4" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="P4" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="Q4" s="22" t="s">
+        <v>308</v>
+      </c>
+      <c r="R4" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="S4" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="T4" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="U4" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="V4" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="W4" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="X4" s="20" t="s">
         <v>312</v>
       </c>
-      <c r="R2" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="S2" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="T2" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="U2" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="V2" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="W2" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="X2" s="20" t="s">
-        <v>319</v>
-      </c>
-      <c r="Y2" s="20" t="s">
-        <v>320</v>
-      </c>
-      <c r="Z2" s="11" t="s">
-        <v>301</v>
-      </c>
-      <c r="AA2" s="21" t="s">
+      <c r="Y4" s="20" t="s">
+        <v>315</v>
+      </c>
+      <c r="Z4" s="11" t="s">
+        <v>300</v>
+      </c>
+      <c r="AA4" s="11" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="5" spans="1:29" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="B5" s="9" t="s">
         <v>302</v>
       </c>
-    </row>
-    <row r="3" spans="1:29" ht="32.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="12" t="s">
-        <v>70</v>
-      </c>
-      <c r="B3" s="9" t="s">
-        <v>75</v>
-      </c>
-      <c r="C3" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="D3" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="E3" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="F3" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="G3" s="12" t="s">
-        <v>80</v>
-      </c>
-      <c r="H3" s="12" t="s">
-        <v>80</v>
-      </c>
-      <c r="I3" s="12" t="s">
-        <v>80</v>
-      </c>
-      <c r="J3" s="12" t="s">
-        <v>80</v>
-      </c>
-      <c r="K3" s="12" t="s">
-        <v>80</v>
-      </c>
-      <c r="L3" s="12" t="s">
-        <v>80</v>
-      </c>
-      <c r="M3" s="12" t="s">
-        <v>80</v>
-      </c>
-      <c r="N3" s="12" t="s">
-        <v>80</v>
-      </c>
-      <c r="O3" s="12" t="s">
-        <v>80</v>
-      </c>
-      <c r="P3" s="12" t="s">
-        <v>80</v>
-      </c>
-      <c r="Q3" s="22" t="s">
+      <c r="C5" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="D5" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="E5" s="16" t="s">
+        <v>303</v>
+      </c>
+      <c r="F5" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="G5" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="H5" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="I5" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="J5" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="K5" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="L5" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="M5" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="N5" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="O5" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="P5" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="Q5" s="22" t="s">
         <v>309</v>
       </c>
-      <c r="R3" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="S3" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="T3" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="U3" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="V3" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="W3" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="X3" s="20" t="s">
+      <c r="R5" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="S5" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="T5" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="U5" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="V5" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="W5" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="X5" s="20" t="s">
         <v>313</v>
-      </c>
-      <c r="Y3" s="20" t="s">
-        <v>316</v>
-      </c>
-      <c r="Z3" s="11" t="s">
-        <v>301</v>
-      </c>
-      <c r="AA3" s="11" t="s">
-        <v>301</v>
-      </c>
-    </row>
-    <row r="4" spans="1:29" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="12" t="s">
-        <v>69</v>
-      </c>
-      <c r="B4" s="9" t="s">
-        <v>303</v>
-      </c>
-      <c r="C4" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="D4" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="E4" s="16" t="s">
-        <v>304</v>
-      </c>
-      <c r="F4" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="G4" s="12" t="s">
-        <v>80</v>
-      </c>
-      <c r="H4" s="12" t="s">
-        <v>80</v>
-      </c>
-      <c r="I4" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="J4" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="K4" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="L4" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="M4" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="N4" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="O4" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="P4" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="Q4" s="22" t="s">
-        <v>310</v>
-      </c>
-      <c r="R4" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="S4" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="T4" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="U4" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="V4" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="W4" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="X4" s="20" t="s">
-        <v>314</v>
-      </c>
-      <c r="Y4" s="20" t="s">
-        <v>318</v>
-      </c>
-      <c r="Z4" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="AA4" s="11" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="5" spans="1:29" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="12" t="s">
-        <v>71</v>
-      </c>
-      <c r="B5" s="9" t="s">
-        <v>76</v>
-      </c>
-      <c r="C5" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="D5" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="E5" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="F5" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="G5" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="H5" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="I5" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="J5" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="K5" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="L5" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="M5" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="N5" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="O5" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="P5" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="Q5" s="20" t="s">
-        <v>311</v>
-      </c>
-      <c r="R5" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="S5" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="T5" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="U5" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="V5" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="W5" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="X5" s="20" t="s">
-        <v>315</v>
       </c>
       <c r="Y5" s="20" t="s">
         <v>317</v>
       </c>
       <c r="Z5" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="AA5" s="11" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="6" spans="1:29" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="D6" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="E6" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="F6" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="G6" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="H6" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="I6" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="J6" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="K6" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="L6" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="M6" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="N6" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="O6" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="P6" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="Q6" s="20" t="s">
+        <v>310</v>
+      </c>
+      <c r="R6" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="S6" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="T6" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="U6" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="V6" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="W6" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="X6" s="20" t="s">
+        <v>314</v>
+      </c>
+      <c r="Y6" s="20" t="s">
+        <v>316</v>
+      </c>
+      <c r="Z6" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="AA6" s="11" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="7" spans="1:29" ht="88.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="13" t="s">
+        <v>72</v>
+      </c>
+      <c r="B7" s="14" t="s">
+        <v>76</v>
+      </c>
+      <c r="C7" s="15" t="s">
+        <v>304</v>
+      </c>
+      <c r="D7" s="15" t="s">
+        <v>304</v>
+      </c>
+      <c r="E7" s="15" t="s">
+        <v>304</v>
+      </c>
+      <c r="F7" s="15" t="s">
+        <v>304</v>
+      </c>
+      <c r="G7" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="H7" s="15" t="s">
+        <v>304</v>
+      </c>
+      <c r="I7" s="15" t="s">
+        <v>304</v>
+      </c>
+      <c r="J7" s="15" t="s">
+        <v>304</v>
+      </c>
+      <c r="K7" s="15" t="s">
+        <v>304</v>
+      </c>
+      <c r="L7" s="15" t="s">
+        <v>304</v>
+      </c>
+      <c r="M7" s="15" t="s">
+        <v>304</v>
+      </c>
+      <c r="N7" s="15" t="s">
+        <v>304</v>
+      </c>
+      <c r="O7" s="15" t="s">
+        <v>304</v>
+      </c>
+      <c r="P7" s="15" t="s">
+        <v>304</v>
+      </c>
+      <c r="Q7" s="20" t="s">
+        <v>320</v>
+      </c>
+      <c r="R7" s="15" t="s">
+        <v>304</v>
+      </c>
+      <c r="S7" s="15" t="s">
+        <v>304</v>
+      </c>
+      <c r="T7" s="15" t="s">
+        <v>304</v>
+      </c>
+      <c r="U7" s="15" t="s">
+        <v>304</v>
+      </c>
+      <c r="V7" s="15" t="s">
+        <v>304</v>
+      </c>
+      <c r="W7" s="15" t="s">
+        <v>304</v>
+      </c>
+      <c r="X7" s="20" t="s">
+        <v>321</v>
+      </c>
+      <c r="Y7" s="20" t="s">
+        <v>322</v>
+      </c>
+      <c r="Z7" s="15" t="s">
+        <v>304</v>
+      </c>
+      <c r="AA7" s="15" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="8" spans="1:29" x14ac:dyDescent="0.3">
+      <c r="A8" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="C8" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="D8" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="E8" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="F8" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="G8" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="H8" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="I8" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="J8" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="K8" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="L8" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="M8" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="N8" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="O8" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="P8" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="Q8" s="20" t="s">
+        <v>326</v>
+      </c>
+      <c r="R8" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="S8" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="T8" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="U8" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="V8" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="W8" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="X8" s="20" t="s">
+        <v>327</v>
+      </c>
+      <c r="Y8" s="20" t="s">
+        <v>328</v>
+      </c>
+      <c r="Z8" s="11" t="s">
+        <v>300</v>
+      </c>
+      <c r="AA8" s="11" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="9" spans="1:29" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="C9" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="AA5" s="11" t="s">
+      <c r="D9" s="4" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="6" spans="1:29" ht="88.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="13" t="s">
-        <v>72</v>
-      </c>
-      <c r="B6" s="14" t="s">
-        <v>77</v>
-      </c>
-      <c r="C6" s="15" t="s">
-        <v>305</v>
-      </c>
-      <c r="D6" s="15" t="s">
-        <v>305</v>
-      </c>
-      <c r="E6" s="15" t="s">
-        <v>305</v>
-      </c>
-      <c r="F6" s="15" t="s">
-        <v>305</v>
-      </c>
-      <c r="G6" s="11" t="s">
+      <c r="E9" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="H6" s="15" t="s">
-        <v>305</v>
-      </c>
-      <c r="I6" s="15" t="s">
-        <v>305</v>
-      </c>
-      <c r="J6" s="15" t="s">
-        <v>305</v>
-      </c>
-      <c r="K6" s="15" t="s">
-        <v>305</v>
-      </c>
-      <c r="L6" s="15" t="s">
-        <v>305</v>
-      </c>
-      <c r="M6" s="15" t="s">
-        <v>305</v>
-      </c>
-      <c r="N6" s="15" t="s">
-        <v>305</v>
-      </c>
-      <c r="O6" s="15" t="s">
-        <v>305</v>
-      </c>
-      <c r="P6" s="15" t="s">
-        <v>305</v>
-      </c>
-      <c r="Q6" s="20" t="s">
-        <v>321</v>
-      </c>
-      <c r="R6" s="15" t="s">
-        <v>305</v>
-      </c>
-      <c r="S6" s="15" t="s">
-        <v>305</v>
-      </c>
-      <c r="T6" s="15" t="s">
-        <v>305</v>
-      </c>
-      <c r="U6" s="15" t="s">
-        <v>305</v>
-      </c>
-      <c r="V6" s="15" t="s">
-        <v>305</v>
-      </c>
-      <c r="W6" s="15" t="s">
-        <v>305</v>
-      </c>
-      <c r="X6" s="20" t="s">
-        <v>322</v>
-      </c>
-      <c r="Y6" s="20" t="s">
+      <c r="F9" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="I9" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="J9" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="K9" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="L9" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="M9" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="N9" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="O9" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="P9" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="Q9" s="20" t="s">
         <v>323</v>
       </c>
-      <c r="Z6" s="15" t="s">
-        <v>305</v>
-      </c>
-      <c r="AA6" s="15" t="s">
-        <v>305</v>
-      </c>
-    </row>
-    <row r="7" spans="1:29" x14ac:dyDescent="0.3">
-      <c r="A7" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="B7" s="9" t="s">
-        <v>78</v>
-      </c>
-      <c r="C7" s="11" t="s">
+      <c r="R9" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="D7" s="11" t="s">
+      <c r="S9" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="E7" s="11" t="s">
+      <c r="T9" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="F7" s="11" t="s">
+      <c r="U9" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="G7" s="11" t="s">
+      <c r="V9" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="H7" s="11" t="s">
+      <c r="W9" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="I7" s="11" t="s">
+      <c r="X9" s="20" t="s">
+        <v>324</v>
+      </c>
+      <c r="Y9" s="20" t="s">
+        <v>325</v>
+      </c>
+      <c r="Z9" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="J7" s="11" t="s">
+      <c r="AA9" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="K7" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="L7" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="M7" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="N7" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="O7" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="P7" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="Q7" s="20" t="s">
-        <v>327</v>
-      </c>
-      <c r="R7" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="S7" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="T7" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="U7" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="V7" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="W7" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="X7" s="20" t="s">
-        <v>328</v>
-      </c>
-      <c r="Y7" s="20" t="s">
-        <v>329</v>
-      </c>
-      <c r="Z7" s="11" t="s">
-        <v>301</v>
-      </c>
-      <c r="AA7" s="11" t="s">
-        <v>301</v>
-      </c>
-    </row>
-    <row r="8" spans="1:29" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="7" t="s">
-        <v>74</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="F8" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="G8" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="H8" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="I8" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="J8" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="K8" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="L8" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="M8" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="N8" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="O8" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="P8" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="Q8" s="20" t="s">
-        <v>324</v>
-      </c>
-      <c r="R8" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="S8" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="T8" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="U8" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="V8" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="W8" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="X8" s="20" t="s">
-        <v>325</v>
-      </c>
-      <c r="Y8" s="20" t="s">
-        <v>326</v>
-      </c>
-      <c r="Z8" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="AA8" s="4" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="9" spans="1:29" x14ac:dyDescent="0.3">
-      <c r="A9" s="7"/>
-      <c r="B9" s="3"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
-      <c r="E9" s="3"/>
-      <c r="F9" s="3"/>
-      <c r="G9" s="3"/>
-      <c r="H9" s="3"/>
-      <c r="I9" s="3"/>
-      <c r="J9" s="3"/>
-      <c r="K9" s="3"/>
-      <c r="L9" s="3"/>
-      <c r="M9" s="3"/>
     </row>
     <row r="10" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A10" s="7"/>
@@ -4230,12 +4313,27 @@
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A28" s="7"/>
+      <c r="B28" s="3"/>
+      <c r="C28" s="3"/>
+      <c r="D28" s="3"/>
+      <c r="E28" s="3"/>
+      <c r="F28" s="3"/>
+      <c r="G28" s="3"/>
+      <c r="H28" s="3"/>
+      <c r="I28" s="3"/>
+      <c r="J28" s="3"/>
+      <c r="K28" s="3"/>
+      <c r="L28" s="3"/>
+      <c r="M28" s="3"/>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A29" s="7"/>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A30" s="7"/>
+    </row>
+    <row r="31" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A31" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Updated Program.cs, newly generated speech files
</commit_message>
<xml_diff>
--- a/SpeechGenerationAudit.xlsx
+++ b/SpeechGenerationAudit.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pc\Speech Generation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA6D698E-4A88-405C-A4C2-895588681F36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7EECFBD-EEEA-4139-94CD-6CB05F3CEF8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{A672C37D-E69E-470F-9024-46D64C3F6E80}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{A672C37D-E69E-470F-9024-46D64C3F6E80}"/>
   </bookViews>
   <sheets>
     <sheet name="Audio + String Table " sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="717" uniqueCount="335">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="716" uniqueCount="334">
   <si>
     <t>Unity Key</t>
   </si>
@@ -282,9 +282,6 @@
     <t xml:space="preserve">Accurate </t>
   </si>
   <si>
-    <t>Need device to check</t>
-  </si>
-  <si>
     <t>Unity Danish Text</t>
   </si>
   <si>
@@ -327,9 +324,6 @@
     <t>¡Fantástico! ¡Podemos disfrutar juntos!</t>
   </si>
   <si>
-    <t xml:space="preserve">Very quick towards the end </t>
-  </si>
-  <si>
     <t>Unity Dutch Text</t>
   </si>
   <si>
@@ -618,15 +612,6 @@
     <t xml:space="preserve">Фантастика! Вы сегодня в отличной форме! </t>
   </si>
   <si>
-    <t xml:space="preserve">Very robotic sound </t>
-  </si>
-  <si>
-    <t>Not a very accurate translation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Audio glitch </t>
-  </si>
-  <si>
     <t>Unity Russian Text</t>
   </si>
   <si>
@@ -960,9 +945,6 @@
     <t xml:space="preserve">Fixed </t>
   </si>
   <si>
-    <t xml:space="preserve">There is Norwegian audio, but not Norwegian text. </t>
-  </si>
-  <si>
     <t>No audio : FIXED</t>
   </si>
   <si>
@@ -1045,13 +1027,28 @@
   </si>
   <si>
     <t>No audio: ปลดล็อกเกมใช่หรือไม่?</t>
+  </si>
+  <si>
+    <t>Very quick towards the end : FIXED</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Very quick towards the end: FIXED </t>
+  </si>
+  <si>
+    <t>Very robotic sound ; FIXED</t>
+  </si>
+  <si>
+    <t>Not a very accurate translation: FIXED</t>
+  </si>
+  <si>
+    <t>Audio glitch: FIXED</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1109,6 +1106,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -1145,7 +1149,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
@@ -1194,9 +1198,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -1211,6 +1212,10 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1610,25 +1615,25 @@
         <v>2</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>252</v>
+        <v>247</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>3</v>
@@ -1640,121 +1645,121 @@
         <v>3</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="N1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="P1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="R1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="T1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="V1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="X1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="Y1" s="1" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="Z1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="AA1" s="1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="AB1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="AC1" s="1" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="AD1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="AE1" s="1" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="AF1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="AG1" s="1" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="AH1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="AI1" s="1" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="AJ1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="AK1" s="1" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="AL1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="AM1" s="1" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
       <c r="AN1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="AO1" s="1" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="AP1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="AQ1" s="1" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
       <c r="AR1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="AS1" s="1" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
       <c r="AT1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="AU1" s="1" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="AV1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="AW1" s="1" t="s">
-        <v>228</v>
+        <v>223</v>
       </c>
       <c r="AX1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="AY1" s="1" t="s">
-        <v>236</v>
+        <v>231</v>
       </c>
       <c r="AZ1" s="1" t="s">
         <v>3</v>
@@ -1768,25 +1773,25 @@
         <v>63</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="D2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="F2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="G2" s="9" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="H2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="I2" s="9" t="s">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="J2" s="10" t="s">
         <v>56</v>
@@ -1798,121 +1803,121 @@
         <v>56</v>
       </c>
       <c r="M2" s="9" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="N2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="O2" s="9" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="P2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="Q2" s="9" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="R2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="S2" s="9" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="T2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="U2" s="9" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="V2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="W2" s="9" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="X2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="Y2" s="9" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="Z2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AA2" s="9" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="AB2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AC2" s="9" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="AD2" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="AE2" s="18" t="s">
-        <v>154</v>
-      </c>
-      <c r="AF2" s="19" t="s">
-        <v>307</v>
+      <c r="AE2" s="24" t="s">
+        <v>152</v>
+      </c>
+      <c r="AF2" s="25" t="s">
+        <v>301</v>
       </c>
       <c r="AG2" s="9" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="AH2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AI2" s="9" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="AJ2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AK2" s="9" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="AL2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AM2" s="9" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="AN2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AO2" s="9" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="AP2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AQ2" s="9" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="AR2" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="AS2" s="18" t="s">
-        <v>212</v>
-      </c>
-      <c r="AT2" s="19" t="s">
-        <v>307</v>
-      </c>
-      <c r="AU2" s="18" t="s">
-        <v>221</v>
-      </c>
-      <c r="AV2" s="19" t="s">
-        <v>307</v>
+      <c r="AS2" s="24" t="s">
+        <v>207</v>
+      </c>
+      <c r="AT2" s="25" t="s">
+        <v>301</v>
+      </c>
+      <c r="AU2" s="24" t="s">
+        <v>216</v>
+      </c>
+      <c r="AV2" s="25" t="s">
+        <v>301</v>
       </c>
       <c r="AW2" s="9" t="s">
-        <v>229</v>
+        <v>224</v>
       </c>
       <c r="AX2" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AY2" s="9" t="s">
-        <v>237</v>
+        <v>232</v>
       </c>
       <c r="AZ2" s="10" t="s">
         <v>56</v>
@@ -1926,25 +1931,25 @@
         <v>64</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="D3" s="10" t="s">
         <v>56</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="F3" s="10" t="s">
         <v>56</v>
       </c>
       <c r="G3" s="9" t="s">
-        <v>257</v>
+        <v>252</v>
       </c>
       <c r="H3" s="10" t="s">
         <v>56</v>
       </c>
       <c r="I3" s="9" t="s">
-        <v>245</v>
+        <v>240</v>
       </c>
       <c r="J3" s="10" t="s">
         <v>56</v>
@@ -1962,115 +1967,115 @@
         <v>56</v>
       </c>
       <c r="O3" s="9" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="P3" s="10" t="s">
         <v>56</v>
       </c>
       <c r="Q3" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="R3" s="10" t="s">
         <v>56</v>
       </c>
       <c r="S3" s="9" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="T3" s="10" t="s">
         <v>56</v>
       </c>
       <c r="U3" s="9" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="V3" s="10" t="s">
         <v>56</v>
       </c>
       <c r="W3" s="9" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="X3" s="10" t="s">
         <v>56</v>
       </c>
       <c r="Y3" s="9" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="Z3" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AA3" s="9" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="AB3" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AC3" s="9" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="AD3" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="AE3" s="18" t="s">
-        <v>155</v>
-      </c>
-      <c r="AF3" s="19" t="s">
-        <v>307</v>
+      <c r="AE3" s="24" t="s">
+        <v>153</v>
+      </c>
+      <c r="AF3" s="25" t="s">
+        <v>301</v>
       </c>
       <c r="AG3" s="9" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="AH3" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AI3" s="9" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="AJ3" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AK3" s="9" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="AL3" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AM3" s="9" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="AN3" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AO3" s="9" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
       <c r="AP3" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AQ3" s="9" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
       <c r="AR3" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="AS3" s="18" t="s">
-        <v>213</v>
-      </c>
-      <c r="AT3" s="19" t="s">
-        <v>307</v>
-      </c>
-      <c r="AU3" s="18" t="s">
-        <v>222</v>
-      </c>
-      <c r="AV3" s="19" t="s">
-        <v>307</v>
+      <c r="AS3" s="24" t="s">
+        <v>208</v>
+      </c>
+      <c r="AT3" s="25" t="s">
+        <v>301</v>
+      </c>
+      <c r="AU3" s="24" t="s">
+        <v>217</v>
+      </c>
+      <c r="AV3" s="25" t="s">
+        <v>301</v>
       </c>
       <c r="AW3" s="9" t="s">
-        <v>230</v>
+        <v>225</v>
       </c>
       <c r="AX3" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AY3" s="9" t="s">
-        <v>238</v>
+        <v>233</v>
       </c>
       <c r="AZ3" s="10" t="s">
         <v>56</v>
@@ -2084,25 +2089,25 @@
         <v>60</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>271</v>
+        <v>266</v>
       </c>
       <c r="D4" s="10" t="s">
         <v>56</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
       <c r="F4" s="10" t="s">
         <v>56</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="H4" s="10" t="s">
         <v>56</v>
       </c>
       <c r="I4" s="9" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
       <c r="J4" s="10" t="s">
         <v>56</v>
@@ -2113,122 +2118,122 @@
       <c r="L4" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="M4" s="23" t="s">
-        <v>84</v>
-      </c>
-      <c r="N4" s="24" t="s">
-        <v>305</v>
+      <c r="M4" s="22" t="s">
+        <v>83</v>
+      </c>
+      <c r="N4" s="23" t="s">
+        <v>300</v>
       </c>
       <c r="O4" s="9" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="P4" s="10" t="s">
         <v>56</v>
       </c>
       <c r="Q4" s="16" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="R4" s="16" t="s">
-        <v>95</v>
+        <v>329</v>
       </c>
       <c r="S4" s="9" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="T4" s="10" t="s">
         <v>56</v>
       </c>
       <c r="U4" s="9" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="V4" s="10" t="s">
         <v>56</v>
       </c>
       <c r="W4" s="9" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="X4" s="10" t="s">
         <v>56</v>
       </c>
       <c r="Y4" s="9" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="Z4" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AA4" s="9" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="AB4" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AC4" s="9" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="AD4" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="AE4" s="18" t="s">
-        <v>156</v>
-      </c>
-      <c r="AF4" s="19" t="s">
-        <v>307</v>
+      <c r="AE4" s="24" t="s">
+        <v>154</v>
+      </c>
+      <c r="AF4" s="25" t="s">
+        <v>301</v>
       </c>
       <c r="AG4" s="9" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="AH4" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AI4" s="9" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="AJ4" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AK4" s="9" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="AL4" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AM4" s="16" t="s">
-        <v>187</v>
-      </c>
-      <c r="AN4" s="17" t="s">
-        <v>192</v>
+        <v>185</v>
+      </c>
+      <c r="AN4" s="16" t="s">
+        <v>331</v>
       </c>
       <c r="AO4" s="9" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
       <c r="AP4" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AQ4" s="9" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
       <c r="AR4" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="AS4" s="18" t="s">
-        <v>214</v>
-      </c>
-      <c r="AT4" s="19" t="s">
-        <v>307</v>
-      </c>
-      <c r="AU4" s="18" t="s">
-        <v>223</v>
-      </c>
-      <c r="AV4" s="19" t="s">
-        <v>307</v>
+      <c r="AS4" s="24" t="s">
+        <v>209</v>
+      </c>
+      <c r="AT4" s="25" t="s">
+        <v>301</v>
+      </c>
+      <c r="AU4" s="24" t="s">
+        <v>218</v>
+      </c>
+      <c r="AV4" s="25" t="s">
+        <v>301</v>
       </c>
       <c r="AW4" s="9" t="s">
-        <v>231</v>
+        <v>226</v>
       </c>
       <c r="AX4" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AY4" s="9" t="s">
-        <v>239</v>
+        <v>234</v>
       </c>
       <c r="AZ4" s="10" t="s">
         <v>56</v>
@@ -2242,25 +2247,25 @@
         <v>57</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>272</v>
+        <v>267</v>
       </c>
       <c r="D5" s="10" t="s">
         <v>56</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
       <c r="F5" s="10" t="s">
         <v>56</v>
       </c>
       <c r="G5" s="9" t="s">
-        <v>261</v>
+        <v>256</v>
       </c>
       <c r="H5" s="10" t="s">
         <v>56</v>
       </c>
       <c r="I5" s="9" t="s">
-        <v>247</v>
+        <v>242</v>
       </c>
       <c r="J5" s="10" t="s">
         <v>56</v>
@@ -2271,122 +2276,122 @@
       <c r="L5" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="M5" s="23" t="s">
-        <v>85</v>
-      </c>
-      <c r="N5" s="24" t="s">
-        <v>305</v>
+      <c r="M5" s="22" t="s">
+        <v>84</v>
+      </c>
+      <c r="N5" s="23" t="s">
+        <v>300</v>
       </c>
       <c r="O5" s="9" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="P5" s="10" t="s">
         <v>56</v>
       </c>
       <c r="Q5" s="9" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="R5" s="10" t="s">
         <v>56</v>
       </c>
       <c r="S5" s="9" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="T5" s="10" t="s">
         <v>56</v>
       </c>
       <c r="U5" s="9" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="V5" s="10" t="s">
         <v>56</v>
       </c>
       <c r="W5" s="9" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="X5" s="10" t="s">
         <v>56</v>
       </c>
       <c r="Y5" s="9" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="Z5" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AA5" s="16" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="AB5" s="16" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="AC5" s="9" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="AD5" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="AE5" s="18" t="s">
-        <v>157</v>
-      </c>
-      <c r="AF5" s="19" t="s">
-        <v>307</v>
+      <c r="AE5" s="24" t="s">
+        <v>155</v>
+      </c>
+      <c r="AF5" s="25" t="s">
+        <v>301</v>
       </c>
       <c r="AG5" s="9" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="AH5" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AI5" s="9" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="AJ5" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AK5" s="9" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="AL5" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AM5" s="16" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="AN5" s="16" t="s">
-        <v>193</v>
+        <v>332</v>
       </c>
       <c r="AO5" s="9" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="AP5" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AQ5" s="9" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="AR5" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="AS5" s="18" t="s">
-        <v>215</v>
-      </c>
-      <c r="AT5" s="19" t="s">
-        <v>307</v>
-      </c>
-      <c r="AU5" s="18" t="s">
-        <v>224</v>
-      </c>
-      <c r="AV5" s="19" t="s">
-        <v>307</v>
+      <c r="AS5" s="24" t="s">
+        <v>210</v>
+      </c>
+      <c r="AT5" s="25" t="s">
+        <v>301</v>
+      </c>
+      <c r="AU5" s="24" t="s">
+        <v>219</v>
+      </c>
+      <c r="AV5" s="25" t="s">
+        <v>301</v>
       </c>
       <c r="AW5" s="9" t="s">
-        <v>232</v>
+        <v>227</v>
       </c>
       <c r="AX5" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AY5" s="9" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="AZ5" s="10" t="s">
         <v>56</v>
@@ -2400,28 +2405,28 @@
         <v>58</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>273</v>
+        <v>268</v>
       </c>
       <c r="D6" s="10" t="s">
         <v>59</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>263</v>
+        <v>258</v>
       </c>
       <c r="F6" s="10" t="s">
         <v>59</v>
       </c>
       <c r="G6" s="9" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="H6" s="10" t="s">
         <v>59</v>
       </c>
       <c r="I6" s="9" t="s">
-        <v>248</v>
+        <v>243</v>
       </c>
       <c r="J6" s="10" t="s">
-        <v>251</v>
+        <v>246</v>
       </c>
       <c r="K6" s="9" t="s">
         <v>34</v>
@@ -2436,115 +2441,115 @@
         <v>59</v>
       </c>
       <c r="O6" s="9" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="P6" s="10" t="s">
         <v>59</v>
       </c>
       <c r="Q6" s="9" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="R6" s="10" t="s">
         <v>59</v>
       </c>
       <c r="S6" s="9" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="T6" s="10" t="s">
         <v>59</v>
       </c>
       <c r="U6" s="9" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="V6" s="10" t="s">
         <v>59</v>
       </c>
       <c r="W6" s="9" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="X6" s="10" t="s">
         <v>59</v>
       </c>
       <c r="Y6" s="9" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="Z6" s="10" t="s">
         <v>59</v>
       </c>
       <c r="AA6" s="16" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="AB6" s="16" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="AC6" s="9" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="AD6" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="AE6" s="18" t="s">
-        <v>158</v>
-      </c>
-      <c r="AF6" s="19" t="s">
-        <v>307</v>
+      <c r="AE6" s="24" t="s">
+        <v>156</v>
+      </c>
+      <c r="AF6" s="25" t="s">
+        <v>301</v>
       </c>
       <c r="AG6" s="9" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="AH6" s="10" t="s">
         <v>59</v>
       </c>
       <c r="AI6" s="9" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="AJ6" s="10" t="s">
         <v>59</v>
       </c>
       <c r="AK6" s="9" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="AL6" s="10" t="s">
         <v>59</v>
       </c>
       <c r="AM6" s="9" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="AN6" s="10" t="s">
         <v>59</v>
       </c>
       <c r="AO6" s="9" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
       <c r="AP6" s="10" t="s">
         <v>59</v>
       </c>
       <c r="AQ6" s="9" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="AR6" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="AS6" s="18" t="s">
-        <v>217</v>
-      </c>
-      <c r="AT6" s="19" t="s">
-        <v>307</v>
-      </c>
-      <c r="AU6" s="18" t="s">
-        <v>225</v>
-      </c>
-      <c r="AV6" s="19" t="s">
-        <v>307</v>
+      <c r="AS6" s="24" t="s">
+        <v>212</v>
+      </c>
+      <c r="AT6" s="25" t="s">
+        <v>301</v>
+      </c>
+      <c r="AU6" s="24" t="s">
+        <v>220</v>
+      </c>
+      <c r="AV6" s="25" t="s">
+        <v>301</v>
       </c>
       <c r="AW6" s="9" t="s">
-        <v>233</v>
+        <v>228</v>
       </c>
       <c r="AX6" s="10" t="s">
         <v>59</v>
       </c>
       <c r="AY6" s="9" t="s">
-        <v>241</v>
+        <v>236</v>
       </c>
       <c r="AZ6" s="10" t="s">
         <v>59</v>
@@ -2558,25 +2563,25 @@
         <v>61</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>274</v>
+        <v>269</v>
       </c>
       <c r="D7" s="10" t="s">
         <v>56</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>264</v>
+        <v>259</v>
       </c>
       <c r="F7" s="10" t="s">
         <v>56</v>
       </c>
       <c r="G7" s="9" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="H7" s="10" t="s">
         <v>56</v>
       </c>
       <c r="I7" s="9" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
       <c r="J7" s="10" t="s">
         <v>56</v>
@@ -2588,121 +2593,121 @@
         <v>56</v>
       </c>
       <c r="M7" s="9" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="N7" s="10" t="s">
         <v>56</v>
       </c>
       <c r="O7" s="9" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="P7" s="10" t="s">
         <v>56</v>
       </c>
       <c r="Q7" s="16" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="R7" s="16" t="s">
-        <v>95</v>
+        <v>330</v>
       </c>
       <c r="S7" s="9" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="T7" s="10" t="s">
         <v>56</v>
       </c>
       <c r="U7" s="9" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="V7" s="10" t="s">
         <v>56</v>
       </c>
       <c r="W7" s="9" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="X7" s="10" t="s">
         <v>56</v>
       </c>
       <c r="Y7" s="9" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="Z7" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AA7" s="16" t="s">
+        <v>140</v>
+      </c>
+      <c r="AB7" s="16" t="s">
         <v>142</v>
       </c>
-      <c r="AB7" s="16" t="s">
-        <v>144</v>
-      </c>
       <c r="AC7" s="9" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="AD7" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="AE7" s="18" t="s">
-        <v>159</v>
-      </c>
-      <c r="AF7" s="19" t="s">
-        <v>307</v>
+      <c r="AE7" s="24" t="s">
+        <v>157</v>
+      </c>
+      <c r="AF7" s="25" t="s">
+        <v>301</v>
       </c>
       <c r="AG7" s="9" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="AH7" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AI7" s="9" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="AJ7" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AK7" s="9" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="AL7" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AM7" s="16" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="AN7" s="17" t="s">
-        <v>194</v>
+        <v>333</v>
       </c>
       <c r="AO7" s="9" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
       <c r="AP7" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AQ7" s="9" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="AR7" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="AS7" s="18" t="s">
-        <v>218</v>
-      </c>
-      <c r="AT7" s="19" t="s">
-        <v>307</v>
-      </c>
-      <c r="AU7" s="18" t="s">
-        <v>226</v>
-      </c>
-      <c r="AV7" s="19" t="s">
-        <v>307</v>
+      <c r="AS7" s="24" t="s">
+        <v>213</v>
+      </c>
+      <c r="AT7" s="25" t="s">
+        <v>301</v>
+      </c>
+      <c r="AU7" s="24" t="s">
+        <v>221</v>
+      </c>
+      <c r="AV7" s="25" t="s">
+        <v>301</v>
       </c>
       <c r="AW7" s="9" t="s">
-        <v>234</v>
+        <v>229</v>
       </c>
       <c r="AX7" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AY7" s="9" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="AZ7" s="10" t="s">
         <v>56</v>
@@ -2716,25 +2721,25 @@
         <v>62</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="D8" s="10" t="s">
         <v>56</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>267</v>
+        <v>262</v>
       </c>
       <c r="F8" s="10" t="s">
         <v>56</v>
       </c>
       <c r="G8" s="9" t="s">
-        <v>266</v>
+        <v>261</v>
       </c>
       <c r="H8" s="10" t="s">
         <v>56</v>
       </c>
       <c r="I8" s="9" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="J8" s="10" t="s">
         <v>56</v>
@@ -2752,115 +2757,115 @@
         <v>56</v>
       </c>
       <c r="O8" s="9" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="P8" s="10" t="s">
         <v>56</v>
       </c>
       <c r="Q8" s="9" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="R8" s="10" t="s">
         <v>56</v>
       </c>
       <c r="S8" s="9" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="T8" s="10" t="s">
         <v>56</v>
       </c>
       <c r="U8" s="9" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="V8" s="10" t="s">
         <v>56</v>
       </c>
       <c r="W8" s="9" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="X8" s="10" t="s">
         <v>56</v>
       </c>
       <c r="Y8" s="9" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="Z8" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AA8" s="9" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="AB8" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AC8" s="9" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="AD8" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="AE8" s="18" t="s">
-        <v>160</v>
-      </c>
-      <c r="AF8" s="19" t="s">
-        <v>307</v>
+      <c r="AE8" s="24" t="s">
+        <v>158</v>
+      </c>
+      <c r="AF8" s="25" t="s">
+        <v>301</v>
       </c>
       <c r="AG8" s="9" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="AH8" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AI8" s="9" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="AJ8" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AK8" s="9" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="AL8" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AM8" s="9" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="AN8" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AO8" s="9" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="AP8" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AQ8" s="9" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="AR8" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="AS8" s="18" t="s">
-        <v>219</v>
-      </c>
-      <c r="AT8" s="19" t="s">
-        <v>307</v>
-      </c>
-      <c r="AU8" s="18" t="s">
-        <v>227</v>
-      </c>
-      <c r="AV8" s="19" t="s">
-        <v>307</v>
+      <c r="AS8" s="24" t="s">
+        <v>214</v>
+      </c>
+      <c r="AT8" s="25" t="s">
+        <v>301</v>
+      </c>
+      <c r="AU8" s="24" t="s">
+        <v>222</v>
+      </c>
+      <c r="AV8" s="25" t="s">
+        <v>301</v>
       </c>
       <c r="AW8" s="9" t="s">
-        <v>235</v>
+        <v>230</v>
       </c>
       <c r="AX8" s="10" t="s">
         <v>56</v>
       </c>
       <c r="AY8" s="9" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
       <c r="AZ8" s="10" t="s">
         <v>56</v>
@@ -2922,9 +2927,7 @@
       <c r="K11" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="AL11" s="19" t="s">
-        <v>306</v>
-      </c>
+      <c r="AL11" s="18"/>
     </row>
     <row r="12" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
@@ -3300,79 +3303,79 @@
         <v>67</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>276</v>
+        <v>271</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>277</v>
+        <v>272</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>278</v>
+        <v>273</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>279</v>
+        <v>274</v>
       </c>
       <c r="G1" s="6" t="s">
         <v>68</v>
       </c>
       <c r="H1" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="I1" s="6" t="s">
+        <v>276</v>
+      </c>
+      <c r="J1" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="K1" s="6" t="s">
+        <v>278</v>
+      </c>
+      <c r="L1" s="6" t="s">
+        <v>279</v>
+      </c>
+      <c r="M1" s="6" t="s">
         <v>280</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="N1" s="6" t="s">
         <v>281</v>
       </c>
-      <c r="J1" s="6" t="s">
+      <c r="O1" s="6" t="s">
         <v>282</v>
       </c>
-      <c r="K1" s="6" t="s">
+      <c r="P1" s="6" t="s">
         <v>283</v>
       </c>
-      <c r="L1" s="6" t="s">
+      <c r="Q1" s="6" t="s">
         <v>284</v>
       </c>
-      <c r="M1" s="6" t="s">
+      <c r="R1" s="6" t="s">
         <v>285</v>
       </c>
-      <c r="N1" s="6" t="s">
+      <c r="S1" s="6" t="s">
         <v>286</v>
       </c>
-      <c r="O1" s="6" t="s">
+      <c r="T1" s="6" t="s">
         <v>287</v>
       </c>
-      <c r="P1" s="6" t="s">
+      <c r="U1" s="6" t="s">
         <v>288</v>
       </c>
-      <c r="Q1" s="6" t="s">
+      <c r="V1" s="6" t="s">
         <v>289</v>
       </c>
-      <c r="R1" s="6" t="s">
+      <c r="W1" s="6" t="s">
         <v>290</v>
       </c>
-      <c r="S1" s="6" t="s">
+      <c r="X1" s="6" t="s">
         <v>291</v>
       </c>
-      <c r="T1" s="6" t="s">
+      <c r="Y1" s="6" t="s">
         <v>292</v>
       </c>
-      <c r="U1" s="6" t="s">
+      <c r="Z1" s="6" t="s">
         <v>293</v>
       </c>
-      <c r="V1" s="6" t="s">
+      <c r="AA1" s="6" t="s">
         <v>294</v>
-      </c>
-      <c r="W1" s="6" t="s">
-        <v>295</v>
-      </c>
-      <c r="X1" s="6" t="s">
-        <v>296</v>
-      </c>
-      <c r="Y1" s="6" t="s">
-        <v>297</v>
-      </c>
-      <c r="Z1" s="6" t="s">
-        <v>298</v>
-      </c>
-      <c r="AA1" s="6" t="s">
-        <v>299</v>
       </c>
       <c r="AB1" s="6"/>
       <c r="AC1" s="6"/>
@@ -3426,8 +3429,8 @@
       <c r="P2" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="Q2" s="22" t="s">
-        <v>311</v>
+      <c r="Q2" s="21" t="s">
+        <v>305</v>
       </c>
       <c r="R2" s="11" t="s">
         <v>79</v>
@@ -3447,17 +3450,17 @@
       <c r="W2" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="X2" s="20" t="s">
-        <v>318</v>
-      </c>
-      <c r="Y2" s="20" t="s">
-        <v>319</v>
+      <c r="X2" s="19" t="s">
+        <v>312</v>
+      </c>
+      <c r="Y2" s="19" t="s">
+        <v>313</v>
       </c>
       <c r="Z2" s="11" t="s">
-        <v>300</v>
-      </c>
-      <c r="AA2" s="21" t="s">
-        <v>301</v>
+        <v>295</v>
+      </c>
+      <c r="AA2" s="20" t="s">
+        <v>296</v>
       </c>
     </row>
     <row r="3" spans="1:29" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -3465,7 +3468,7 @@
         <v>70</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>331</v>
+        <v>325</v>
       </c>
       <c r="C3" s="11" t="s">
         <v>79</v>
@@ -3509,8 +3512,8 @@
       <c r="P3" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="Q3" s="22" t="s">
-        <v>332</v>
+      <c r="Q3" s="21" t="s">
+        <v>326</v>
       </c>
       <c r="R3" s="11" t="s">
         <v>79</v>
@@ -3530,25 +3533,25 @@
       <c r="W3" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="X3" s="20" t="s">
-        <v>333</v>
-      </c>
-      <c r="Y3" s="20" t="s">
-        <v>334</v>
+      <c r="X3" s="19" t="s">
+        <v>327</v>
+      </c>
+      <c r="Y3" s="19" t="s">
+        <v>328</v>
       </c>
       <c r="Z3" s="11" t="s">
-        <v>300</v>
+        <v>295</v>
       </c>
       <c r="AA3" s="11" t="s">
-        <v>300</v>
+        <v>295</v>
       </c>
     </row>
     <row r="4" spans="1:29" ht="32.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="12" t="s">
-        <v>329</v>
+        <v>323</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>330</v>
+        <v>324</v>
       </c>
       <c r="C4" s="11" t="s">
         <v>79</v>
@@ -3592,8 +3595,8 @@
       <c r="P4" s="12" t="s">
         <v>79</v>
       </c>
-      <c r="Q4" s="22" t="s">
-        <v>308</v>
+      <c r="Q4" s="21" t="s">
+        <v>302</v>
       </c>
       <c r="R4" s="11" t="s">
         <v>79</v>
@@ -3613,17 +3616,17 @@
       <c r="W4" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="X4" s="20" t="s">
-        <v>312</v>
-      </c>
-      <c r="Y4" s="20" t="s">
-        <v>315</v>
+      <c r="X4" s="19" t="s">
+        <v>306</v>
+      </c>
+      <c r="Y4" s="19" t="s">
+        <v>309</v>
       </c>
       <c r="Z4" s="11" t="s">
-        <v>300</v>
+        <v>295</v>
       </c>
       <c r="AA4" s="11" t="s">
-        <v>300</v>
+        <v>295</v>
       </c>
     </row>
     <row r="5" spans="1:29" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -3631,7 +3634,7 @@
         <v>69</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>302</v>
+        <v>297</v>
       </c>
       <c r="C5" s="11" t="s">
         <v>79</v>
@@ -3640,44 +3643,44 @@
         <v>79</v>
       </c>
       <c r="E5" s="16" t="s">
+        <v>298</v>
+      </c>
+      <c r="F5" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="G5" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="H5" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="I5" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="J5" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="K5" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="L5" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="M5" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="N5" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="O5" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="P5" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="Q5" s="21" t="s">
         <v>303</v>
       </c>
-      <c r="F5" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="G5" s="12" t="s">
-        <v>79</v>
-      </c>
-      <c r="H5" s="12" t="s">
-        <v>79</v>
-      </c>
-      <c r="I5" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="J5" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="K5" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="L5" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="M5" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="N5" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="O5" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="P5" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="Q5" s="22" t="s">
-        <v>309</v>
-      </c>
       <c r="R5" s="11" t="s">
         <v>79</v>
       </c>
@@ -3696,11 +3699,11 @@
       <c r="W5" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="X5" s="20" t="s">
-        <v>313</v>
-      </c>
-      <c r="Y5" s="20" t="s">
-        <v>317</v>
+      <c r="X5" s="19" t="s">
+        <v>307</v>
+      </c>
+      <c r="Y5" s="19" t="s">
+        <v>311</v>
       </c>
       <c r="Z5" s="11" t="s">
         <v>79</v>
@@ -3758,32 +3761,32 @@
       <c r="P6" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="Q6" s="20" t="s">
+      <c r="Q6" s="19" t="s">
+        <v>304</v>
+      </c>
+      <c r="R6" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="S6" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="T6" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="U6" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="V6" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="W6" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="X6" s="19" t="s">
+        <v>308</v>
+      </c>
+      <c r="Y6" s="19" t="s">
         <v>310</v>
-      </c>
-      <c r="R6" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="S6" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="T6" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="U6" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="V6" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="W6" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="X6" s="20" t="s">
-        <v>314</v>
-      </c>
-      <c r="Y6" s="20" t="s">
-        <v>316</v>
       </c>
       <c r="Z6" s="11" t="s">
         <v>79</v>
@@ -3800,79 +3803,79 @@
         <v>76</v>
       </c>
       <c r="C7" s="15" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="D7" s="15" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="E7" s="15" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="F7" s="15" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="G7" s="11" t="s">
         <v>79</v>
       </c>
       <c r="H7" s="15" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="I7" s="15" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="J7" s="15" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="K7" s="15" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="L7" s="15" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="M7" s="15" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="N7" s="15" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="O7" s="15" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="P7" s="15" t="s">
-        <v>304</v>
-      </c>
-      <c r="Q7" s="20" t="s">
-        <v>320</v>
+        <v>299</v>
+      </c>
+      <c r="Q7" s="19" t="s">
+        <v>314</v>
       </c>
       <c r="R7" s="15" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="S7" s="15" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="T7" s="15" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="U7" s="15" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="V7" s="15" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="W7" s="15" t="s">
-        <v>304</v>
-      </c>
-      <c r="X7" s="20" t="s">
-        <v>321</v>
-      </c>
-      <c r="Y7" s="20" t="s">
-        <v>322</v>
+        <v>299</v>
+      </c>
+      <c r="X7" s="19" t="s">
+        <v>315</v>
+      </c>
+      <c r="Y7" s="19" t="s">
+        <v>316</v>
       </c>
       <c r="Z7" s="15" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="AA7" s="15" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
     </row>
     <row r="8" spans="1:29" x14ac:dyDescent="0.3">
@@ -3924,8 +3927,8 @@
       <c r="P8" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="Q8" s="20" t="s">
-        <v>326</v>
+      <c r="Q8" s="19" t="s">
+        <v>320</v>
       </c>
       <c r="R8" s="11" t="s">
         <v>79</v>
@@ -3945,100 +3948,100 @@
       <c r="W8" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="X8" s="20" t="s">
-        <v>327</v>
-      </c>
-      <c r="Y8" s="20" t="s">
-        <v>328</v>
+      <c r="X8" s="19" t="s">
+        <v>321</v>
+      </c>
+      <c r="Y8" s="19" t="s">
+        <v>322</v>
       </c>
       <c r="Z8" s="11" t="s">
-        <v>300</v>
+        <v>295</v>
       </c>
       <c r="AA8" s="11" t="s">
-        <v>300</v>
+        <v>295</v>
       </c>
     </row>
     <row r="9" spans="1:29" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="7" t="s">
+      <c r="A9" s="12" t="s">
         <v>74</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="C9" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="F9" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="G9" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="H9" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="I9" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="J9" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="K9" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="L9" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="M9" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="N9" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="O9" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="P9" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="Q9" s="20" t="s">
-        <v>323</v>
-      </c>
-      <c r="R9" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="S9" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="T9" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="U9" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="V9" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="W9" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="X9" s="20" t="s">
-        <v>324</v>
-      </c>
-      <c r="Y9" s="20" t="s">
-        <v>325</v>
-      </c>
-      <c r="Z9" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="AA9" s="4" t="s">
-        <v>80</v>
+      <c r="C9" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="D9" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="E9" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="F9" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="G9" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="H9" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="I9" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="J9" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="K9" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="L9" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="M9" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="N9" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="O9" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="P9" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="Q9" s="19" t="s">
+        <v>317</v>
+      </c>
+      <c r="R9" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="S9" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="T9" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="U9" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="V9" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="W9" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="X9" s="19" t="s">
+        <v>318</v>
+      </c>
+      <c r="Y9" s="19" t="s">
+        <v>319</v>
+      </c>
+      <c r="Z9" s="11" t="s">
+        <v>295</v>
+      </c>
+      <c r="AA9" s="11" t="s">
+        <v>295</v>
       </c>
     </row>
     <row r="10" spans="1:29" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Updated speech, newly generated prompt
</commit_message>
<xml_diff>
--- a/SpeechGenerationAudit.xlsx
+++ b/SpeechGenerationAudit.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pc\Speech Generation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7EECFBD-EEEA-4139-94CD-6CB05F3CEF8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCF64BA9-137C-410A-A51D-C71DA63CB00E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{A672C37D-E69E-470F-9024-46D64C3F6E80}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{A672C37D-E69E-470F-9024-46D64C3F6E80}"/>
   </bookViews>
   <sheets>
     <sheet name="Audio + String Table " sheetId="1" r:id="rId1"/>
@@ -939,9 +939,6 @@
     <t>Same meaning, different words</t>
   </si>
   <si>
-    <t xml:space="preserve">Audio matches filename, doesn't match r written (heading is just "Take a break", subheading is German speech prompt translated) </t>
-  </si>
-  <si>
     <t xml:space="preserve">Fixed </t>
   </si>
   <si>
@@ -1042,13 +1039,16 @@
   </si>
   <si>
     <t>Audio glitch: FIXED</t>
+  </si>
+  <si>
+    <t>Audio matches filename, doesn't match r written (heading is just "Take a break", subheading is German speech prompt translated) : FIXED</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1074,13 +1074,6 @@
     <font>
       <sz val="11"/>
       <color rgb="FF00B050"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="8" tint="0.39997558519241921"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1149,7 +1142,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
@@ -1185,37 +1178,31 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1856,11 +1843,11 @@
       <c r="AD2" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="AE2" s="24" t="s">
+      <c r="AE2" s="21" t="s">
         <v>152</v>
       </c>
-      <c r="AF2" s="25" t="s">
-        <v>301</v>
+      <c r="AF2" s="22" t="s">
+        <v>300</v>
       </c>
       <c r="AG2" s="9" t="s">
         <v>160</v>
@@ -1898,17 +1885,17 @@
       <c r="AR2" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="AS2" s="24" t="s">
+      <c r="AS2" s="21" t="s">
         <v>207</v>
       </c>
-      <c r="AT2" s="25" t="s">
-        <v>301</v>
-      </c>
-      <c r="AU2" s="24" t="s">
+      <c r="AT2" s="22" t="s">
+        <v>300</v>
+      </c>
+      <c r="AU2" s="21" t="s">
         <v>216</v>
       </c>
-      <c r="AV2" s="25" t="s">
-        <v>301</v>
+      <c r="AV2" s="22" t="s">
+        <v>300</v>
       </c>
       <c r="AW2" s="9" t="s">
         <v>224</v>
@@ -2014,11 +2001,11 @@
       <c r="AD3" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="AE3" s="24" t="s">
+      <c r="AE3" s="21" t="s">
         <v>153</v>
       </c>
-      <c r="AF3" s="25" t="s">
-        <v>301</v>
+      <c r="AF3" s="22" t="s">
+        <v>300</v>
       </c>
       <c r="AG3" s="9" t="s">
         <v>161</v>
@@ -2056,17 +2043,17 @@
       <c r="AR3" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="AS3" s="24" t="s">
+      <c r="AS3" s="21" t="s">
         <v>208</v>
       </c>
-      <c r="AT3" s="25" t="s">
-        <v>301</v>
-      </c>
-      <c r="AU3" s="24" t="s">
+      <c r="AT3" s="22" t="s">
+        <v>300</v>
+      </c>
+      <c r="AU3" s="21" t="s">
         <v>217</v>
       </c>
-      <c r="AV3" s="25" t="s">
-        <v>301</v>
+      <c r="AV3" s="22" t="s">
+        <v>300</v>
       </c>
       <c r="AW3" s="9" t="s">
         <v>225</v>
@@ -2118,11 +2105,11 @@
       <c r="L4" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="M4" s="22" t="s">
+      <c r="M4" s="19" t="s">
         <v>83</v>
       </c>
-      <c r="N4" s="23" t="s">
-        <v>300</v>
+      <c r="N4" s="20" t="s">
+        <v>299</v>
       </c>
       <c r="O4" s="9" t="s">
         <v>97</v>
@@ -2130,11 +2117,11 @@
       <c r="P4" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="Q4" s="16" t="s">
+      <c r="Q4" s="13" t="s">
         <v>89</v>
       </c>
-      <c r="R4" s="16" t="s">
-        <v>329</v>
+      <c r="R4" s="13" t="s">
+        <v>328</v>
       </c>
       <c r="S4" s="9" t="s">
         <v>105</v>
@@ -2172,11 +2159,11 @@
       <c r="AD4" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="AE4" s="24" t="s">
+      <c r="AE4" s="21" t="s">
         <v>154</v>
       </c>
-      <c r="AF4" s="25" t="s">
-        <v>301</v>
+      <c r="AF4" s="22" t="s">
+        <v>300</v>
       </c>
       <c r="AG4" s="9" t="s">
         <v>162</v>
@@ -2196,11 +2183,11 @@
       <c r="AL4" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="AM4" s="16" t="s">
+      <c r="AM4" s="13" t="s">
         <v>185</v>
       </c>
-      <c r="AN4" s="16" t="s">
-        <v>331</v>
+      <c r="AN4" s="13" t="s">
+        <v>330</v>
       </c>
       <c r="AO4" s="9" t="s">
         <v>194</v>
@@ -2214,17 +2201,17 @@
       <c r="AR4" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="AS4" s="24" t="s">
+      <c r="AS4" s="21" t="s">
         <v>209</v>
       </c>
-      <c r="AT4" s="25" t="s">
-        <v>301</v>
-      </c>
-      <c r="AU4" s="24" t="s">
+      <c r="AT4" s="22" t="s">
+        <v>300</v>
+      </c>
+      <c r="AU4" s="21" t="s">
         <v>218</v>
       </c>
-      <c r="AV4" s="25" t="s">
-        <v>301</v>
+      <c r="AV4" s="22" t="s">
+        <v>300</v>
       </c>
       <c r="AW4" s="9" t="s">
         <v>226</v>
@@ -2276,11 +2263,11 @@
       <c r="L5" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="M5" s="22" t="s">
+      <c r="M5" s="19" t="s">
         <v>84</v>
       </c>
-      <c r="N5" s="23" t="s">
-        <v>300</v>
+      <c r="N5" s="20" t="s">
+        <v>299</v>
       </c>
       <c r="O5" s="9" t="s">
         <v>98</v>
@@ -2318,10 +2305,10 @@
       <c r="Z5" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="AA5" s="16" t="s">
+      <c r="AA5" s="13" t="s">
         <v>138</v>
       </c>
-      <c r="AB5" s="16" t="s">
+      <c r="AB5" s="13" t="s">
         <v>142</v>
       </c>
       <c r="AC5" s="9" t="s">
@@ -2330,11 +2317,11 @@
       <c r="AD5" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="AE5" s="24" t="s">
+      <c r="AE5" s="21" t="s">
         <v>155</v>
       </c>
-      <c r="AF5" s="25" t="s">
-        <v>301</v>
+      <c r="AF5" s="22" t="s">
+        <v>300</v>
       </c>
       <c r="AG5" s="9" t="s">
         <v>163</v>
@@ -2354,11 +2341,11 @@
       <c r="AL5" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="AM5" s="16" t="s">
+      <c r="AM5" s="13" t="s">
         <v>186</v>
       </c>
-      <c r="AN5" s="16" t="s">
-        <v>332</v>
+      <c r="AN5" s="13" t="s">
+        <v>331</v>
       </c>
       <c r="AO5" s="9" t="s">
         <v>195</v>
@@ -2372,17 +2359,17 @@
       <c r="AR5" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="AS5" s="24" t="s">
+      <c r="AS5" s="21" t="s">
         <v>210</v>
       </c>
-      <c r="AT5" s="25" t="s">
-        <v>301</v>
-      </c>
-      <c r="AU5" s="24" t="s">
+      <c r="AT5" s="22" t="s">
+        <v>300</v>
+      </c>
+      <c r="AU5" s="21" t="s">
         <v>219</v>
       </c>
-      <c r="AV5" s="25" t="s">
-        <v>301</v>
+      <c r="AV5" s="22" t="s">
+        <v>300</v>
       </c>
       <c r="AW5" s="9" t="s">
         <v>227</v>
@@ -2476,10 +2463,10 @@
       <c r="Z6" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="AA6" s="16" t="s">
+      <c r="AA6" s="13" t="s">
         <v>139</v>
       </c>
-      <c r="AB6" s="16" t="s">
+      <c r="AB6" s="13" t="s">
         <v>142</v>
       </c>
       <c r="AC6" s="9" t="s">
@@ -2488,11 +2475,11 @@
       <c r="AD6" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="AE6" s="24" t="s">
+      <c r="AE6" s="21" t="s">
         <v>156</v>
       </c>
-      <c r="AF6" s="25" t="s">
-        <v>301</v>
+      <c r="AF6" s="22" t="s">
+        <v>300</v>
       </c>
       <c r="AG6" s="9" t="s">
         <v>164</v>
@@ -2530,17 +2517,17 @@
       <c r="AR6" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="AS6" s="24" t="s">
+      <c r="AS6" s="21" t="s">
         <v>212</v>
       </c>
-      <c r="AT6" s="25" t="s">
-        <v>301</v>
-      </c>
-      <c r="AU6" s="24" t="s">
+      <c r="AT6" s="22" t="s">
+        <v>300</v>
+      </c>
+      <c r="AU6" s="21" t="s">
         <v>220</v>
       </c>
-      <c r="AV6" s="25" t="s">
-        <v>301</v>
+      <c r="AV6" s="22" t="s">
+        <v>300</v>
       </c>
       <c r="AW6" s="9" t="s">
         <v>228</v>
@@ -2604,11 +2591,11 @@
       <c r="P7" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="Q7" s="16" t="s">
+      <c r="Q7" s="13" t="s">
         <v>92</v>
       </c>
-      <c r="R7" s="16" t="s">
-        <v>330</v>
+      <c r="R7" s="13" t="s">
+        <v>329</v>
       </c>
       <c r="S7" s="9" t="s">
         <v>108</v>
@@ -2634,10 +2621,10 @@
       <c r="Z7" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="AA7" s="16" t="s">
+      <c r="AA7" s="13" t="s">
         <v>140</v>
       </c>
-      <c r="AB7" s="16" t="s">
+      <c r="AB7" s="13" t="s">
         <v>142</v>
       </c>
       <c r="AC7" s="9" t="s">
@@ -2646,11 +2633,11 @@
       <c r="AD7" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="AE7" s="24" t="s">
+      <c r="AE7" s="21" t="s">
         <v>157</v>
       </c>
-      <c r="AF7" s="25" t="s">
-        <v>301</v>
+      <c r="AF7" s="22" t="s">
+        <v>300</v>
       </c>
       <c r="AG7" s="9" t="s">
         <v>165</v>
@@ -2670,11 +2657,11 @@
       <c r="AL7" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="AM7" s="16" t="s">
+      <c r="AM7" s="13" t="s">
         <v>187</v>
       </c>
-      <c r="AN7" s="17" t="s">
-        <v>333</v>
+      <c r="AN7" s="14" t="s">
+        <v>332</v>
       </c>
       <c r="AO7" s="9" t="s">
         <v>197</v>
@@ -2688,17 +2675,17 @@
       <c r="AR7" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="AS7" s="24" t="s">
+      <c r="AS7" s="21" t="s">
         <v>213</v>
       </c>
-      <c r="AT7" s="25" t="s">
-        <v>301</v>
-      </c>
-      <c r="AU7" s="24" t="s">
+      <c r="AT7" s="22" t="s">
+        <v>300</v>
+      </c>
+      <c r="AU7" s="21" t="s">
         <v>221</v>
       </c>
-      <c r="AV7" s="25" t="s">
-        <v>301</v>
+      <c r="AV7" s="22" t="s">
+        <v>300</v>
       </c>
       <c r="AW7" s="9" t="s">
         <v>229</v>
@@ -2804,11 +2791,11 @@
       <c r="AD8" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="AE8" s="24" t="s">
+      <c r="AE8" s="21" t="s">
         <v>158</v>
       </c>
-      <c r="AF8" s="25" t="s">
-        <v>301</v>
+      <c r="AF8" s="22" t="s">
+        <v>300</v>
       </c>
       <c r="AG8" s="9" t="s">
         <v>166</v>
@@ -2846,17 +2833,17 @@
       <c r="AR8" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="AS8" s="24" t="s">
+      <c r="AS8" s="21" t="s">
         <v>214</v>
       </c>
-      <c r="AT8" s="25" t="s">
-        <v>301</v>
-      </c>
-      <c r="AU8" s="24" t="s">
+      <c r="AT8" s="22" t="s">
+        <v>300</v>
+      </c>
+      <c r="AU8" s="21" t="s">
         <v>222</v>
       </c>
-      <c r="AV8" s="25" t="s">
-        <v>301</v>
+      <c r="AV8" s="22" t="s">
+        <v>300</v>
       </c>
       <c r="AW8" s="9" t="s">
         <v>230</v>
@@ -2927,7 +2914,7 @@
       <c r="K11" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="AL11" s="18"/>
+      <c r="AL11" s="15"/>
     </row>
     <row r="12" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
@@ -3429,8 +3416,8 @@
       <c r="P2" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="Q2" s="21" t="s">
-        <v>305</v>
+      <c r="Q2" s="18" t="s">
+        <v>304</v>
       </c>
       <c r="R2" s="11" t="s">
         <v>79</v>
@@ -3450,16 +3437,16 @@
       <c r="W2" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="X2" s="19" t="s">
+      <c r="X2" s="16" t="s">
+        <v>311</v>
+      </c>
+      <c r="Y2" s="16" t="s">
         <v>312</v>
-      </c>
-      <c r="Y2" s="19" t="s">
-        <v>313</v>
       </c>
       <c r="Z2" s="11" t="s">
         <v>295</v>
       </c>
-      <c r="AA2" s="20" t="s">
+      <c r="AA2" s="17" t="s">
         <v>296</v>
       </c>
     </row>
@@ -3468,76 +3455,76 @@
         <v>70</v>
       </c>
       <c r="B3" s="9" t="s">
+        <v>324</v>
+      </c>
+      <c r="C3" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="D3" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="E3" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="F3" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="G3" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="H3" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="I3" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="J3" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="K3" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="L3" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="M3" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="N3" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="O3" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="P3" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="Q3" s="18" t="s">
         <v>325</v>
       </c>
-      <c r="C3" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="D3" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="E3" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="F3" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="G3" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="H3" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="I3" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="J3" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="K3" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="L3" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="M3" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="N3" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="O3" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="P3" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="Q3" s="21" t="s">
+      <c r="R3" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="S3" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="T3" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="U3" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="V3" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="W3" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="X3" s="16" t="s">
         <v>326</v>
       </c>
-      <c r="R3" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="S3" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="T3" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="U3" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="V3" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="W3" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="X3" s="19" t="s">
+      <c r="Y3" s="16" t="s">
         <v>327</v>
-      </c>
-      <c r="Y3" s="19" t="s">
-        <v>328</v>
       </c>
       <c r="Z3" s="11" t="s">
         <v>295</v>
@@ -3548,11 +3535,11 @@
     </row>
     <row r="4" spans="1:29" ht="32.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="12" t="s">
+        <v>322</v>
+      </c>
+      <c r="B4" s="9" t="s">
         <v>323</v>
       </c>
-      <c r="B4" s="9" t="s">
-        <v>324</v>
-      </c>
       <c r="C4" s="11" t="s">
         <v>79</v>
       </c>
@@ -3595,8 +3582,8 @@
       <c r="P4" s="12" t="s">
         <v>79</v>
       </c>
-      <c r="Q4" s="21" t="s">
-        <v>302</v>
+      <c r="Q4" s="18" t="s">
+        <v>301</v>
       </c>
       <c r="R4" s="11" t="s">
         <v>79</v>
@@ -3616,11 +3603,11 @@
       <c r="W4" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="X4" s="19" t="s">
-        <v>306</v>
-      </c>
-      <c r="Y4" s="19" t="s">
-        <v>309</v>
+      <c r="X4" s="16" t="s">
+        <v>305</v>
+      </c>
+      <c r="Y4" s="16" t="s">
+        <v>308</v>
       </c>
       <c r="Z4" s="11" t="s">
         <v>295</v>
@@ -3642,7 +3629,7 @@
       <c r="D5" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="E5" s="16" t="s">
+      <c r="E5" s="13" t="s">
         <v>298</v>
       </c>
       <c r="F5" s="11" t="s">
@@ -3678,8 +3665,8 @@
       <c r="P5" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="Q5" s="21" t="s">
-        <v>303</v>
+      <c r="Q5" s="18" t="s">
+        <v>302</v>
       </c>
       <c r="R5" s="11" t="s">
         <v>79</v>
@@ -3699,11 +3686,11 @@
       <c r="W5" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="X5" s="19" t="s">
-        <v>307</v>
-      </c>
-      <c r="Y5" s="19" t="s">
-        <v>311</v>
+      <c r="X5" s="16" t="s">
+        <v>306</v>
+      </c>
+      <c r="Y5" s="16" t="s">
+        <v>310</v>
       </c>
       <c r="Z5" s="11" t="s">
         <v>79</v>
@@ -3761,8 +3748,8 @@
       <c r="P6" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="Q6" s="19" t="s">
-        <v>304</v>
+      <c r="Q6" s="16" t="s">
+        <v>303</v>
       </c>
       <c r="R6" s="11" t="s">
         <v>79</v>
@@ -3782,11 +3769,11 @@
       <c r="W6" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="X6" s="19" t="s">
-        <v>308</v>
-      </c>
-      <c r="Y6" s="19" t="s">
-        <v>310</v>
+      <c r="X6" s="16" t="s">
+        <v>307</v>
+      </c>
+      <c r="Y6" s="16" t="s">
+        <v>309</v>
       </c>
       <c r="Z6" s="11" t="s">
         <v>79</v>
@@ -3796,86 +3783,86 @@
       </c>
     </row>
     <row r="7" spans="1:29" ht="88.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="13" t="s">
+      <c r="A7" s="23" t="s">
         <v>72</v>
       </c>
-      <c r="B7" s="14" t="s">
+      <c r="B7" s="13" t="s">
         <v>76</v>
       </c>
-      <c r="C7" s="15" t="s">
-        <v>299</v>
-      </c>
-      <c r="D7" s="15" t="s">
-        <v>299</v>
-      </c>
-      <c r="E7" s="15" t="s">
-        <v>299</v>
-      </c>
-      <c r="F7" s="15" t="s">
-        <v>299</v>
-      </c>
-      <c r="G7" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="H7" s="15" t="s">
-        <v>299</v>
-      </c>
-      <c r="I7" s="15" t="s">
-        <v>299</v>
-      </c>
-      <c r="J7" s="15" t="s">
-        <v>299</v>
-      </c>
-      <c r="K7" s="15" t="s">
-        <v>299</v>
-      </c>
-      <c r="L7" s="15" t="s">
-        <v>299</v>
-      </c>
-      <c r="M7" s="15" t="s">
-        <v>299</v>
-      </c>
-      <c r="N7" s="15" t="s">
-        <v>299</v>
-      </c>
-      <c r="O7" s="15" t="s">
-        <v>299</v>
-      </c>
-      <c r="P7" s="15" t="s">
-        <v>299</v>
-      </c>
-      <c r="Q7" s="19" t="s">
+      <c r="C7" s="17" t="s">
+        <v>333</v>
+      </c>
+      <c r="D7" s="17" t="s">
+        <v>333</v>
+      </c>
+      <c r="E7" s="17" t="s">
+        <v>333</v>
+      </c>
+      <c r="F7" s="17" t="s">
+        <v>333</v>
+      </c>
+      <c r="G7" s="17" t="s">
+        <v>333</v>
+      </c>
+      <c r="H7" s="17" t="s">
+        <v>333</v>
+      </c>
+      <c r="I7" s="17" t="s">
+        <v>333</v>
+      </c>
+      <c r="J7" s="17" t="s">
+        <v>333</v>
+      </c>
+      <c r="K7" s="17" t="s">
+        <v>333</v>
+      </c>
+      <c r="L7" s="17" t="s">
+        <v>333</v>
+      </c>
+      <c r="M7" s="17" t="s">
+        <v>333</v>
+      </c>
+      <c r="N7" s="17" t="s">
+        <v>333</v>
+      </c>
+      <c r="O7" s="17" t="s">
+        <v>333</v>
+      </c>
+      <c r="P7" s="17" t="s">
+        <v>333</v>
+      </c>
+      <c r="Q7" s="16" t="s">
+        <v>313</v>
+      </c>
+      <c r="R7" s="17" t="s">
+        <v>333</v>
+      </c>
+      <c r="S7" s="17" t="s">
+        <v>333</v>
+      </c>
+      <c r="T7" s="17" t="s">
+        <v>333</v>
+      </c>
+      <c r="U7" s="17" t="s">
+        <v>333</v>
+      </c>
+      <c r="V7" s="17" t="s">
+        <v>333</v>
+      </c>
+      <c r="W7" s="17" t="s">
+        <v>333</v>
+      </c>
+      <c r="X7" s="16" t="s">
         <v>314</v>
       </c>
-      <c r="R7" s="15" t="s">
-        <v>299</v>
-      </c>
-      <c r="S7" s="15" t="s">
-        <v>299</v>
-      </c>
-      <c r="T7" s="15" t="s">
-        <v>299</v>
-      </c>
-      <c r="U7" s="15" t="s">
-        <v>299</v>
-      </c>
-      <c r="V7" s="15" t="s">
-        <v>299</v>
-      </c>
-      <c r="W7" s="15" t="s">
-        <v>299</v>
-      </c>
-      <c r="X7" s="19" t="s">
+      <c r="Y7" s="16" t="s">
         <v>315</v>
       </c>
-      <c r="Y7" s="19" t="s">
-        <v>316</v>
-      </c>
-      <c r="Z7" s="15" t="s">
-        <v>299</v>
-      </c>
-      <c r="AA7" s="15" t="s">
-        <v>299</v>
+      <c r="Z7" s="17" t="s">
+        <v>333</v>
+      </c>
+      <c r="AA7" s="17" t="s">
+        <v>333</v>
       </c>
     </row>
     <row r="8" spans="1:29" x14ac:dyDescent="0.3">
@@ -3927,32 +3914,32 @@
       <c r="P8" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="Q8" s="19" t="s">
+      <c r="Q8" s="16" t="s">
+        <v>319</v>
+      </c>
+      <c r="R8" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="S8" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="T8" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="U8" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="V8" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="W8" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="X8" s="16" t="s">
         <v>320</v>
       </c>
-      <c r="R8" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="S8" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="T8" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="U8" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="V8" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="W8" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="X8" s="19" t="s">
+      <c r="Y8" s="16" t="s">
         <v>321</v>
-      </c>
-      <c r="Y8" s="19" t="s">
-        <v>322</v>
       </c>
       <c r="Z8" s="11" t="s">
         <v>295</v>
@@ -4010,32 +3997,32 @@
       <c r="P9" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="Q9" s="19" t="s">
+      <c r="Q9" s="16" t="s">
+        <v>316</v>
+      </c>
+      <c r="R9" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="S9" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="T9" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="U9" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="V9" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="W9" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="X9" s="16" t="s">
         <v>317</v>
       </c>
-      <c r="R9" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="S9" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="T9" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="U9" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="V9" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="W9" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="X9" s="19" t="s">
+      <c r="Y9" s="16" t="s">
         <v>318</v>
-      </c>
-      <c r="Y9" s="19" t="s">
-        <v>319</v>
       </c>
       <c r="Z9" s="11" t="s">
         <v>295</v>

</xml_diff>

<commit_message>
Improved audio files and adjusted Program.cs
</commit_message>
<xml_diff>
--- a/SpeechGenerationAudit.xlsx
+++ b/SpeechGenerationAudit.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pc\Speech Generation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCF64BA9-137C-410A-A51D-C71DA63CB00E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78409F21-3044-4A76-ACBB-AFD95EE796D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{A672C37D-E69E-470F-9024-46D64C3F6E80}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{A672C37D-E69E-470F-9024-46D64C3F6E80}"/>
   </bookViews>
   <sheets>
     <sheet name="Audio + String Table " sheetId="1" r:id="rId1"/>
@@ -1048,7 +1048,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1106,6 +1106,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF7030A0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -1142,7 +1149,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
@@ -1181,17 +1188,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -1200,9 +1197,16 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1843,10 +1847,10 @@
       <c r="AD2" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="AE2" s="21" t="s">
+      <c r="AE2" s="17" t="s">
         <v>152</v>
       </c>
-      <c r="AF2" s="22" t="s">
+      <c r="AF2" s="18" t="s">
         <v>300</v>
       </c>
       <c r="AG2" s="9" t="s">
@@ -1885,16 +1889,16 @@
       <c r="AR2" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="AS2" s="21" t="s">
+      <c r="AS2" s="17" t="s">
         <v>207</v>
       </c>
-      <c r="AT2" s="22" t="s">
+      <c r="AT2" s="18" t="s">
         <v>300</v>
       </c>
-      <c r="AU2" s="21" t="s">
+      <c r="AU2" s="17" t="s">
         <v>216</v>
       </c>
-      <c r="AV2" s="22" t="s">
+      <c r="AV2" s="18" t="s">
         <v>300</v>
       </c>
       <c r="AW2" s="9" t="s">
@@ -2001,10 +2005,10 @@
       <c r="AD3" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="AE3" s="21" t="s">
+      <c r="AE3" s="17" t="s">
         <v>153</v>
       </c>
-      <c r="AF3" s="22" t="s">
+      <c r="AF3" s="18" t="s">
         <v>300</v>
       </c>
       <c r="AG3" s="9" t="s">
@@ -2043,16 +2047,16 @@
       <c r="AR3" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="AS3" s="21" t="s">
+      <c r="AS3" s="17" t="s">
         <v>208</v>
       </c>
-      <c r="AT3" s="22" t="s">
+      <c r="AT3" s="18" t="s">
         <v>300</v>
       </c>
-      <c r="AU3" s="21" t="s">
+      <c r="AU3" s="17" t="s">
         <v>217</v>
       </c>
-      <c r="AV3" s="22" t="s">
+      <c r="AV3" s="18" t="s">
         <v>300</v>
       </c>
       <c r="AW3" s="9" t="s">
@@ -2105,10 +2109,10 @@
       <c r="L4" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="M4" s="19" t="s">
+      <c r="M4" s="15" t="s">
         <v>83</v>
       </c>
-      <c r="N4" s="20" t="s">
+      <c r="N4" s="16" t="s">
         <v>299</v>
       </c>
       <c r="O4" s="9" t="s">
@@ -2117,10 +2121,10 @@
       <c r="P4" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="Q4" s="13" t="s">
+      <c r="Q4" s="21" t="s">
         <v>89</v>
       </c>
-      <c r="R4" s="13" t="s">
+      <c r="R4" s="21" t="s">
         <v>328</v>
       </c>
       <c r="S4" s="9" t="s">
@@ -2159,10 +2163,10 @@
       <c r="AD4" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="AE4" s="21" t="s">
+      <c r="AE4" s="17" t="s">
         <v>154</v>
       </c>
-      <c r="AF4" s="22" t="s">
+      <c r="AF4" s="18" t="s">
         <v>300</v>
       </c>
       <c r="AG4" s="9" t="s">
@@ -2183,10 +2187,10 @@
       <c r="AL4" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="AM4" s="13" t="s">
+      <c r="AM4" s="21" t="s">
         <v>185</v>
       </c>
-      <c r="AN4" s="13" t="s">
+      <c r="AN4" s="21" t="s">
         <v>330</v>
       </c>
       <c r="AO4" s="9" t="s">
@@ -2201,16 +2205,16 @@
       <c r="AR4" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="AS4" s="21" t="s">
+      <c r="AS4" s="17" t="s">
         <v>209</v>
       </c>
-      <c r="AT4" s="22" t="s">
+      <c r="AT4" s="18" t="s">
         <v>300</v>
       </c>
-      <c r="AU4" s="21" t="s">
+      <c r="AU4" s="17" t="s">
         <v>218</v>
       </c>
-      <c r="AV4" s="22" t="s">
+      <c r="AV4" s="18" t="s">
         <v>300</v>
       </c>
       <c r="AW4" s="9" t="s">
@@ -2263,10 +2267,10 @@
       <c r="L5" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="M5" s="19" t="s">
+      <c r="M5" s="15" t="s">
         <v>84</v>
       </c>
-      <c r="N5" s="20" t="s">
+      <c r="N5" s="16" t="s">
         <v>299</v>
       </c>
       <c r="O5" s="9" t="s">
@@ -2305,10 +2309,10 @@
       <c r="Z5" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="AA5" s="13" t="s">
+      <c r="AA5" s="21" t="s">
         <v>138</v>
       </c>
-      <c r="AB5" s="13" t="s">
+      <c r="AB5" s="21" t="s">
         <v>142</v>
       </c>
       <c r="AC5" s="9" t="s">
@@ -2317,10 +2321,10 @@
       <c r="AD5" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="AE5" s="21" t="s">
+      <c r="AE5" s="17" t="s">
         <v>155</v>
       </c>
-      <c r="AF5" s="22" t="s">
+      <c r="AF5" s="18" t="s">
         <v>300</v>
       </c>
       <c r="AG5" s="9" t="s">
@@ -2341,10 +2345,10 @@
       <c r="AL5" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="AM5" s="13" t="s">
+      <c r="AM5" s="21" t="s">
         <v>186</v>
       </c>
-      <c r="AN5" s="13" t="s">
+      <c r="AN5" s="21" t="s">
         <v>331</v>
       </c>
       <c r="AO5" s="9" t="s">
@@ -2359,16 +2363,16 @@
       <c r="AR5" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="AS5" s="21" t="s">
+      <c r="AS5" s="17" t="s">
         <v>210</v>
       </c>
-      <c r="AT5" s="22" t="s">
+      <c r="AT5" s="18" t="s">
         <v>300</v>
       </c>
-      <c r="AU5" s="21" t="s">
+      <c r="AU5" s="17" t="s">
         <v>219</v>
       </c>
-      <c r="AV5" s="22" t="s">
+      <c r="AV5" s="18" t="s">
         <v>300</v>
       </c>
       <c r="AW5" s="9" t="s">
@@ -2463,10 +2467,10 @@
       <c r="Z6" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="AA6" s="13" t="s">
+      <c r="AA6" s="21" t="s">
         <v>139</v>
       </c>
-      <c r="AB6" s="13" t="s">
+      <c r="AB6" s="21" t="s">
         <v>142</v>
       </c>
       <c r="AC6" s="9" t="s">
@@ -2475,10 +2479,10 @@
       <c r="AD6" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="AE6" s="21" t="s">
+      <c r="AE6" s="17" t="s">
         <v>156</v>
       </c>
-      <c r="AF6" s="22" t="s">
+      <c r="AF6" s="18" t="s">
         <v>300</v>
       </c>
       <c r="AG6" s="9" t="s">
@@ -2517,16 +2521,16 @@
       <c r="AR6" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="AS6" s="21" t="s">
+      <c r="AS6" s="17" t="s">
         <v>212</v>
       </c>
-      <c r="AT6" s="22" t="s">
+      <c r="AT6" s="18" t="s">
         <v>300</v>
       </c>
-      <c r="AU6" s="21" t="s">
+      <c r="AU6" s="17" t="s">
         <v>220</v>
       </c>
-      <c r="AV6" s="22" t="s">
+      <c r="AV6" s="18" t="s">
         <v>300</v>
       </c>
       <c r="AW6" s="9" t="s">
@@ -2591,10 +2595,10 @@
       <c r="P7" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="Q7" s="13" t="s">
+      <c r="Q7" s="21" t="s">
         <v>92</v>
       </c>
-      <c r="R7" s="13" t="s">
+      <c r="R7" s="21" t="s">
         <v>329</v>
       </c>
       <c r="S7" s="9" t="s">
@@ -2621,10 +2625,10 @@
       <c r="Z7" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="AA7" s="13" t="s">
+      <c r="AA7" s="21" t="s">
         <v>140</v>
       </c>
-      <c r="AB7" s="13" t="s">
+      <c r="AB7" s="21" t="s">
         <v>142</v>
       </c>
       <c r="AC7" s="9" t="s">
@@ -2633,10 +2637,10 @@
       <c r="AD7" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="AE7" s="21" t="s">
+      <c r="AE7" s="17" t="s">
         <v>157</v>
       </c>
-      <c r="AF7" s="22" t="s">
+      <c r="AF7" s="18" t="s">
         <v>300</v>
       </c>
       <c r="AG7" s="9" t="s">
@@ -2657,10 +2661,10 @@
       <c r="AL7" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="AM7" s="13" t="s">
+      <c r="AM7" s="21" t="s">
         <v>187</v>
       </c>
-      <c r="AN7" s="14" t="s">
+      <c r="AN7" s="22" t="s">
         <v>332</v>
       </c>
       <c r="AO7" s="9" t="s">
@@ -2675,16 +2679,16 @@
       <c r="AR7" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="AS7" s="21" t="s">
+      <c r="AS7" s="17" t="s">
         <v>213</v>
       </c>
-      <c r="AT7" s="22" t="s">
+      <c r="AT7" s="18" t="s">
         <v>300</v>
       </c>
-      <c r="AU7" s="21" t="s">
+      <c r="AU7" s="17" t="s">
         <v>221</v>
       </c>
-      <c r="AV7" s="22" t="s">
+      <c r="AV7" s="18" t="s">
         <v>300</v>
       </c>
       <c r="AW7" s="9" t="s">
@@ -2791,10 +2795,10 @@
       <c r="AD8" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="AE8" s="21" t="s">
+      <c r="AE8" s="17" t="s">
         <v>158</v>
       </c>
-      <c r="AF8" s="22" t="s">
+      <c r="AF8" s="18" t="s">
         <v>300</v>
       </c>
       <c r="AG8" s="9" t="s">
@@ -2833,16 +2837,16 @@
       <c r="AR8" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="AS8" s="21" t="s">
+      <c r="AS8" s="17" t="s">
         <v>214</v>
       </c>
-      <c r="AT8" s="22" t="s">
+      <c r="AT8" s="18" t="s">
         <v>300</v>
       </c>
-      <c r="AU8" s="21" t="s">
+      <c r="AU8" s="17" t="s">
         <v>222</v>
       </c>
-      <c r="AV8" s="22" t="s">
+      <c r="AV8" s="18" t="s">
         <v>300</v>
       </c>
       <c r="AW8" s="9" t="s">
@@ -2914,7 +2918,7 @@
       <c r="K11" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="AL11" s="15"/>
+      <c r="AL11" s="14"/>
     </row>
     <row r="12" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
@@ -3416,7 +3420,7 @@
       <c r="P2" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="Q2" s="18" t="s">
+      <c r="Q2" s="20" t="s">
         <v>304</v>
       </c>
       <c r="R2" s="11" t="s">
@@ -3437,16 +3441,16 @@
       <c r="W2" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="X2" s="16" t="s">
+      <c r="X2" s="19" t="s">
         <v>311</v>
       </c>
-      <c r="Y2" s="16" t="s">
+      <c r="Y2" s="19" t="s">
         <v>312</v>
       </c>
       <c r="Z2" s="11" t="s">
         <v>295</v>
       </c>
-      <c r="AA2" s="17" t="s">
+      <c r="AA2" s="19" t="s">
         <v>296</v>
       </c>
     </row>
@@ -3499,7 +3503,7 @@
       <c r="P3" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="Q3" s="18" t="s">
+      <c r="Q3" s="20" t="s">
         <v>325</v>
       </c>
       <c r="R3" s="11" t="s">
@@ -3520,10 +3524,10 @@
       <c r="W3" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="X3" s="16" t="s">
+      <c r="X3" s="19" t="s">
         <v>326</v>
       </c>
-      <c r="Y3" s="16" t="s">
+      <c r="Y3" s="19" t="s">
         <v>327</v>
       </c>
       <c r="Z3" s="11" t="s">
@@ -3582,7 +3586,7 @@
       <c r="P4" s="12" t="s">
         <v>79</v>
       </c>
-      <c r="Q4" s="18" t="s">
+      <c r="Q4" s="20" t="s">
         <v>301</v>
       </c>
       <c r="R4" s="11" t="s">
@@ -3603,10 +3607,10 @@
       <c r="W4" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="X4" s="16" t="s">
+      <c r="X4" s="19" t="s">
         <v>305</v>
       </c>
-      <c r="Y4" s="16" t="s">
+      <c r="Y4" s="19" t="s">
         <v>308</v>
       </c>
       <c r="Z4" s="11" t="s">
@@ -3665,7 +3669,7 @@
       <c r="P5" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="Q5" s="18" t="s">
+      <c r="Q5" s="20" t="s">
         <v>302</v>
       </c>
       <c r="R5" s="11" t="s">
@@ -3686,10 +3690,10 @@
       <c r="W5" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="X5" s="16" t="s">
+      <c r="X5" s="19" t="s">
         <v>306</v>
       </c>
-      <c r="Y5" s="16" t="s">
+      <c r="Y5" s="19" t="s">
         <v>310</v>
       </c>
       <c r="Z5" s="11" t="s">
@@ -3748,7 +3752,7 @@
       <c r="P6" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="Q6" s="16" t="s">
+      <c r="Q6" s="19" t="s">
         <v>303</v>
       </c>
       <c r="R6" s="11" t="s">
@@ -3769,10 +3773,10 @@
       <c r="W6" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="X6" s="16" t="s">
+      <c r="X6" s="19" t="s">
         <v>307</v>
       </c>
-      <c r="Y6" s="16" t="s">
+      <c r="Y6" s="19" t="s">
         <v>309</v>
       </c>
       <c r="Z6" s="11" t="s">
@@ -3783,85 +3787,85 @@
       </c>
     </row>
     <row r="7" spans="1:29" ht="88.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="23" t="s">
+      <c r="A7" s="20" t="s">
         <v>72</v>
       </c>
-      <c r="B7" s="13" t="s">
+      <c r="B7" s="21" t="s">
         <v>76</v>
       </c>
-      <c r="C7" s="17" t="s">
+      <c r="C7" s="19" t="s">
         <v>333</v>
       </c>
-      <c r="D7" s="17" t="s">
+      <c r="D7" s="19" t="s">
         <v>333</v>
       </c>
-      <c r="E7" s="17" t="s">
+      <c r="E7" s="19" t="s">
         <v>333</v>
       </c>
-      <c r="F7" s="17" t="s">
+      <c r="F7" s="19" t="s">
         <v>333</v>
       </c>
-      <c r="G7" s="17" t="s">
+      <c r="G7" s="19" t="s">
         <v>333</v>
       </c>
-      <c r="H7" s="17" t="s">
+      <c r="H7" s="19" t="s">
         <v>333</v>
       </c>
-      <c r="I7" s="17" t="s">
+      <c r="I7" s="19" t="s">
         <v>333</v>
       </c>
-      <c r="J7" s="17" t="s">
+      <c r="J7" s="19" t="s">
         <v>333</v>
       </c>
-      <c r="K7" s="17" t="s">
+      <c r="K7" s="19" t="s">
         <v>333</v>
       </c>
-      <c r="L7" s="17" t="s">
+      <c r="L7" s="19" t="s">
         <v>333</v>
       </c>
-      <c r="M7" s="17" t="s">
+      <c r="M7" s="19" t="s">
         <v>333</v>
       </c>
-      <c r="N7" s="17" t="s">
+      <c r="N7" s="19" t="s">
         <v>333</v>
       </c>
-      <c r="O7" s="17" t="s">
+      <c r="O7" s="19" t="s">
         <v>333</v>
       </c>
-      <c r="P7" s="17" t="s">
+      <c r="P7" s="19" t="s">
         <v>333</v>
       </c>
-      <c r="Q7" s="16" t="s">
+      <c r="Q7" s="19" t="s">
         <v>313</v>
       </c>
-      <c r="R7" s="17" t="s">
+      <c r="R7" s="19" t="s">
         <v>333</v>
       </c>
-      <c r="S7" s="17" t="s">
+      <c r="S7" s="19" t="s">
         <v>333</v>
       </c>
-      <c r="T7" s="17" t="s">
+      <c r="T7" s="19" t="s">
         <v>333</v>
       </c>
-      <c r="U7" s="17" t="s">
+      <c r="U7" s="19" t="s">
         <v>333</v>
       </c>
-      <c r="V7" s="17" t="s">
+      <c r="V7" s="19" t="s">
         <v>333</v>
       </c>
-      <c r="W7" s="17" t="s">
+      <c r="W7" s="19" t="s">
         <v>333</v>
       </c>
-      <c r="X7" s="16" t="s">
+      <c r="X7" s="19" t="s">
         <v>314</v>
       </c>
-      <c r="Y7" s="16" t="s">
+      <c r="Y7" s="19" t="s">
         <v>315</v>
       </c>
-      <c r="Z7" s="17" t="s">
+      <c r="Z7" s="19" t="s">
         <v>333</v>
       </c>
-      <c r="AA7" s="17" t="s">
+      <c r="AA7" s="19" t="s">
         <v>333</v>
       </c>
     </row>
@@ -3914,7 +3918,7 @@
       <c r="P8" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="Q8" s="16" t="s">
+      <c r="Q8" s="19" t="s">
         <v>319</v>
       </c>
       <c r="R8" s="11" t="s">
@@ -3935,10 +3939,10 @@
       <c r="W8" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="X8" s="16" t="s">
+      <c r="X8" s="19" t="s">
         <v>320</v>
       </c>
-      <c r="Y8" s="16" t="s">
+      <c r="Y8" s="19" t="s">
         <v>321</v>
       </c>
       <c r="Z8" s="11" t="s">
@@ -3997,7 +4001,7 @@
       <c r="P9" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="Q9" s="16" t="s">
+      <c r="Q9" s="19" t="s">
         <v>316</v>
       </c>
       <c r="R9" s="11" t="s">
@@ -4018,10 +4022,10 @@
       <c r="W9" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="X9" s="16" t="s">
+      <c r="X9" s="19" t="s">
         <v>317</v>
       </c>
-      <c r="Y9" s="16" t="s">
+      <c r="Y9" s="19" t="s">
         <v>318</v>
       </c>
       <c r="Z9" s="11" t="s">

</xml_diff>